<commit_message>
Replace local source paths with public links
</commit_message>
<xml_diff>
--- a/data/reports/personal-ai-compute-report-card.xlsx
+++ b/data/reports/personal-ai-compute-report-card.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R39020c00e1cb428d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compute Report Card" sheetId="2" r:id="R9d241550df324d0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="3" r:id="Rc10bc933a7e149aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R163ee4ffbee94053"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" r:id="Rb0adb89e26b24bcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rb5b5cff3236340b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R19591d2a46124484"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compute Report Card" sheetId="2" r:id="R1767f8bb4cd74ae3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="3" r:id="Rc814db2c664b4b11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Raa0fb099fb4a49af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" r:id="R80b96e0166d64c88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R5ec55904f11b46b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -470,7 +470,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R601f64523c9b4a20"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re8a21602029f46ae"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -522,7 +522,7 @@
     <x:tableColumn id="2" name="Publisher"/>
     <x:tableColumn id="3" name="Title / dataset"/>
     <x:tableColumn id="4" name="Updated / accessed"/>
-    <x:tableColumn id="5" name="URL / path"/>
+    <x:tableColumn id="5" name="Public URL"/>
     <x:tableColumn id="6" name="Use and limitation"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1453,7 +1453,7 @@
     <x:mergeCell ref="B44:N44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18c746c677bb4929"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd85e3ab4f3a54440"/>
 </x:worksheet>
 </file>
 
@@ -3654,7 +3654,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bc03cc0a0f04316"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac8ba386eaa9469a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4707,7 +4707,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7c688171d1342e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09fdb693ea1e44ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4799,7 +4799,7 @@
         <x:v>Updated / accessed</x:v>
       </x:c>
       <x:c r="E5" s="13" t="str">
-        <x:v>URL / path</x:v>
+        <x:v>Public URL</x:v>
       </x:c>
       <x:c r="F5" s="13" t="str">
         <x:v>Use and limitation</x:v>
@@ -4885,7 +4885,7 @@
         <x:v>Model uses the user-specified rounded estimate of 342.8M residents; the selected target is 50%, or 171.4M users</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+    <x:row r="10" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A10" s="17" t="str">
         <x:v>SRC-005</x:v>
       </x:c>
@@ -4893,13 +4893,13 @@
         <x:v>Personal AI forecast</x:v>
       </x:c>
       <x:c r="C10" s="17" t="str">
-        <x:v>System capability and data-center buildouts workbook</x:v>
+        <x:v>Report-card calculation contract</x:v>
       </x:c>
       <x:c r="D10" s="20" t="n">
         <x:v>46260</x:v>
       </x:c>
       <x:c r="E10" s="17" t="str">
-        <x:v>data/reports/legacy/personal-ai-system-capability-and-data-center-buildouts.xlsx</x:v>
+        <x:v>https://github.com/buwilliams/diffuse-personal-ai/blob/main/intent/02-model/06-report-card-calculations.md</x:v>
       </x:c>
       <x:c r="F10" s="17" t="str">
         <x:v>Serving envelope and high-autonomy token mix; assumptions remain editable</x:v>
@@ -4913,13 +4913,13 @@
         <x:v>Personal AI forecast</x:v>
       </x:c>
       <x:c r="C11" s="17" t="str">
-        <x:v>Model-harness capability report card</x:v>
+        <x:v>Model-harness capability report card — HTML</x:v>
       </x:c>
       <x:c r="D11" s="20" t="n">
         <x:v>46260</x:v>
       </x:c>
       <x:c r="E11" s="17" t="str">
-        <x:v>data/reports/personal-ai-four-year-capability-report-card.xlsx</x:v>
+        <x:v>https://diffuse-personal-ai-countdown.buddywilliams.chatgpt.site/?report=capability</x:v>
       </x:c>
       <x:c r="F11" s="17" t="str">
         <x:v>Capability crosses 60% by interpolation around 2027-10-08</x:v>
@@ -4932,7 +4932,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d5467c917f341da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c71e88d68d84bc2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Audit forecast data and projection model
</commit_message>
<xml_diff>
--- a/data/reports/personal-ai-compute-report-card.xlsx
+++ b/data/reports/personal-ai-compute-report-card.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R19591d2a46124484"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compute Report Card" sheetId="2" r:id="R1767f8bb4cd74ae3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="3" r:id="Rc814db2c664b4b11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Raa0fb099fb4a49af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" r:id="R80b96e0166d64c88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R5ec55904f11b46b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2655e89dff2343af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compute Report Card" sheetId="2" r:id="R77f515a337244c5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="3" r:id="R25796c800c7c470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R80aaaa569da04f06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" r:id="R125e40b3a190432c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rc68bc68b5a1c4fb4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -194,13 +194,16 @@
     <x:xf numFmtId="206" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="207" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="208" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="206" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -260,9 +263,6 @@
     <x:xf numFmtId="202" fontId="6" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="202" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
@@ -298,7 +298,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>U.S. serving capacity reaches the threshold in 2027</a:t>
+              <a:t>Published U.S. buildout pipeline reaches the threshold in 2028</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -470,7 +470,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re8a21602029f46ae"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8a28e480823e4a78"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -501,13 +501,13 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="USComputeObservationsTable" displayName="USComputeObservationsTable" ref="A5:G16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="USComputeCapacityInputsTable" displayName="USComputeCapacityInputsTable" ref="A5:G25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Quarter index"/>
     <x:tableColumn id="2" name="Quarter"/>
     <x:tableColumn id="3" name="Cutoff date"/>
     <x:tableColumn id="4" name="U.S. operational H100e"/>
-    <x:tableColumn id="5" name="Operational sites"/>
+    <x:tableColumn id="5" name="Included sites"/>
     <x:tableColumn id="6" name="Evidence class"/>
     <x:tableColumn id="7" name="Source URL"/>
   </x:tableColumns>
@@ -901,13 +901,13 @@
       <x:c r="I5" s="9" t="str">
         <x:v>SUPPORTED USERS</x:v>
       </x:c>
-      <x:c r="J5" s="48" t="str">
+      <x:c r="J5" s="49" t="str">
         <x:v>SUPPLY CROSSING</x:v>
       </x:c>
-      <x:c r="K5" s="48" t="str">
+      <x:c r="K5" s="49" t="str">
         <x:v>SUPPLY CROSSING</x:v>
       </x:c>
-      <x:c r="L5" s="48" t="str">
+      <x:c r="L5" s="49" t="str">
         <x:v>SUPPLY CROSSING</x:v>
       </x:c>
       <x:c r="M5" s="9" t="str">
@@ -918,25 +918,25 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="54" t="n">
+      <x:c r="A6" s="55" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
         <x:v>0.37587725229616675</x:v>
       </x:c>
-      <x:c r="D6" s="55" t="n">
+      <x:c r="D6" s="56" t="n">
         <x:f>'Quarterly Model'!E16</x:f>
         <x:v>13524006</x:v>
       </x:c>
-      <x:c r="E6" s="56"/>
-      <x:c r="F6" s="56"/>
-      <x:c r="G6" s="55" t="n">
+      <x:c r="E6" s="57"/>
+      <x:c r="F6" s="57"/>
+      <x:c r="G6" s="56" t="n">
         <x:f>'Quarterly Model'!I16</x:f>
         <x:v>64425361.043562986</x:v>
       </x:c>
-      <x:c r="J6" s="57" t="n">
+      <x:c r="J6" s="58" t="n">
         <x:f>'Assumptions'!B32</x:f>
-        <x:v>46632.108708204854</x:v>
-      </x:c>
-      <x:c r="M6" s="53" t="str">
+        <x:v>46829.09207929863</x:v>
+      </x:c>
+      <x:c r="M6" s="54" t="str">
         <x:f>'Quarterly Model'!L16</x:f>
         <x:v>F</x:v>
       </x:c>
@@ -992,11 +992,11 @@
       <x:c r="B13" s="17" t="str">
         <x:v>Capability report ≥60%</x:v>
       </x:c>
-      <x:c r="C13" s="29" t="n">
-        <x:v>0.475454716275</x:v>
+      <x:c r="C13" s="31" t="n">
+        <x:v>0.45660533834944794</x:v>
       </x:c>
       <x:c r="D13" s="20" t="n">
-        <x:v>46668</x:v>
+        <x:v>46924</x:v>
       </x:c>
       <x:c r="E13" s="17" t="str">
         <x:v>Waiting</x:v>
@@ -1012,13 +1012,13 @@
       <x:c r="B14" s="17" t="str">
         <x:v>Serve 50% of U.S. population</x:v>
       </x:c>
-      <x:c r="C14" s="29" t="n">
+      <x:c r="C14" s="31" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
         <x:v>0.37587725229616675</x:v>
       </x:c>
       <x:c r="D14" s="20" t="n">
         <x:f>'Assumptions'!B32</x:f>
-        <x:v>46632.108708204854</x:v>
+        <x:v>46829.09207929863</x:v>
       </x:c>
       <x:c r="E14" s="17" t="str">
         <x:v>Waiting</x:v>
@@ -1037,7 +1037,7 @@
       <x:c r="C15" s="24"/>
       <x:c r="D15" s="59" t="n">
         <x:f>'Assumptions'!B35</x:f>
-        <x:v>46668</x:v>
+        <x:v>46924</x:v>
       </x:c>
       <x:c r="E15" s="24" t="str">
         <x:v>Later crossing</x:v>
@@ -1231,7 +1231,7 @@
       </x:c>
       <x:c r="B31" s="19" t="n">
         <x:f>'Quarterly Model'!J17</x:f>
-        <x:v>0.5038169880198742</x:v>
+        <x:v>0.48359766611943783</x:v>
       </x:c>
       <x:c r="C31" s="19" t="n">
         <x:f>1</x:f>
@@ -1245,7 +1245,7 @@
       </x:c>
       <x:c r="B32" s="19" t="n">
         <x:f>'Quarterly Model'!J18</x:f>
-        <x:v>0.660890709854224</x:v>
+        <x:v>0.5660964606872011</x:v>
       </x:c>
       <x:c r="C32" s="19" t="n">
         <x:f>1</x:f>
@@ -1259,7 +1259,7 @@
       </x:c>
       <x:c r="B33" s="19" t="n">
         <x:f>'Quarterly Model'!J19</x:f>
-        <x:v>0.8484310673527545</x:v>
+        <x:v>0.5958694611740921</x:v>
       </x:c>
       <x:c r="C33" s="19" t="n">
         <x:f>1</x:f>
@@ -1273,7 +1273,7 @@
       </x:c>
       <x:c r="B34" s="19" t="n">
         <x:f>'Quarterly Model'!J20</x:f>
-        <x:v>1</x:v>
+        <x:v>0.6459829039518208</x:v>
       </x:c>
       <x:c r="C34" s="19" t="n">
         <x:f>1</x:f>
@@ -1287,7 +1287,7 @@
       </x:c>
       <x:c r="B35" s="19" t="n">
         <x:f>'Quarterly Model'!J21</x:f>
-        <x:v>1</x:v>
+        <x:v>0.8354035263994427</x:v>
       </x:c>
       <x:c r="C35" s="19" t="n">
         <x:f>1</x:f>
@@ -1376,7 +1376,7 @@
         <x:v>Projection</x:v>
       </x:c>
       <x:c r="B42" s="17" t="str">
-        <x:v>Quarterly log-capacity growth is smoothed with a rate trend: the slope of observed growth rates supplies acceleration; the fitted current rate supplies velocity.</x:v>
+        <x:v>The base path sums dated expected or projected operating states in Epoch's current U.S. buildout timeline. The displayed acceleration is descriptive of that source path, not a fitted causal law.</x:v>
       </x:c>
       <x:c r="C42" s="17"/>
       <x:c r="D42" s="17"/>
@@ -1416,7 +1416,7 @@
         <x:v>Caution</x:v>
       </x:c>
       <x:c r="B44" s="17" t="str">
-        <x:v>Epoch estimates carry quantity and timing uncertainty; workload tokens, inference allocation, utilization, active parameters, and overhead are editable assumptions rather than observations.</x:v>
+        <x:v>Epoch covers publicly tracked large sites rather than the full U.S. fleet. Project timing and quantity are uncertain. The editable base case allocates 100% of modeled inference supply to this personal-AI cohort.</x:v>
       </x:c>
       <x:c r="C44" s="17"/>
       <x:c r="D44" s="17"/>
@@ -1453,7 +1453,7 @@
     <x:mergeCell ref="B44:N44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd85e3ab4f3a54440"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf63d864810a34034"/>
 </x:worksheet>
 </file>
 
@@ -2022,58 +2022,58 @@
       <x:c r="X4" s="13" t="str">
         <x:v>2026-Q3</x:v>
       </x:c>
-      <x:c r="Y4" s="35" t="str">
+      <x:c r="Y4" s="36" t="str">
         <x:v>2026-Q4</x:v>
       </x:c>
-      <x:c r="Z4" s="35" t="str">
+      <x:c r="Z4" s="36" t="str">
         <x:v>2026-Q4</x:v>
       </x:c>
-      <x:c r="AA4" s="35" t="str">
+      <x:c r="AA4" s="36" t="str">
         <x:v>2027-Q1</x:v>
       </x:c>
-      <x:c r="AB4" s="35" t="str">
+      <x:c r="AB4" s="36" t="str">
         <x:v>2027-Q1</x:v>
       </x:c>
-      <x:c r="AC4" s="35" t="str">
+      <x:c r="AC4" s="36" t="str">
         <x:v>2027-Q2</x:v>
       </x:c>
-      <x:c r="AD4" s="35" t="str">
+      <x:c r="AD4" s="36" t="str">
         <x:v>2027-Q2</x:v>
       </x:c>
-      <x:c r="AE4" s="35" t="str">
+      <x:c r="AE4" s="36" t="str">
         <x:v>2027-Q3</x:v>
       </x:c>
-      <x:c r="AF4" s="35" t="str">
+      <x:c r="AF4" s="36" t="str">
         <x:v>2027-Q3</x:v>
       </x:c>
-      <x:c r="AG4" s="35" t="str">
+      <x:c r="AG4" s="36" t="str">
         <x:v>2027-Q4</x:v>
       </x:c>
-      <x:c r="AH4" s="35" t="str">
+      <x:c r="AH4" s="36" t="str">
         <x:v>2027-Q4</x:v>
       </x:c>
-      <x:c r="AI4" s="35" t="str">
+      <x:c r="AI4" s="36" t="str">
         <x:v>2028-Q1</x:v>
       </x:c>
-      <x:c r="AJ4" s="35" t="str">
+      <x:c r="AJ4" s="36" t="str">
         <x:v>2028-Q1</x:v>
       </x:c>
-      <x:c r="AK4" s="35" t="str">
+      <x:c r="AK4" s="36" t="str">
         <x:v>2028-Q2</x:v>
       </x:c>
-      <x:c r="AL4" s="35" t="str">
+      <x:c r="AL4" s="36" t="str">
         <x:v>2028-Q2</x:v>
       </x:c>
-      <x:c r="AM4" s="35" t="str">
+      <x:c r="AM4" s="36" t="str">
         <x:v>2028-Q3</x:v>
       </x:c>
-      <x:c r="AN4" s="35" t="str">
+      <x:c r="AN4" s="36" t="str">
         <x:v>2028-Q3</x:v>
       </x:c>
-      <x:c r="AO4" s="35" t="str">
+      <x:c r="AO4" s="36" t="str">
         <x:v>2028-Q4</x:v>
       </x:c>
-      <x:c r="AP4" s="35" t="str">
+      <x:c r="AP4" s="36" t="str">
         <x:v>2028-Q4</x:v>
       </x:c>
       <x:c r="AQ4" s="13" t="str">
@@ -2164,58 +2164,58 @@
       <x:c r="X5" s="13" t="str">
         <x:v>Rate</x:v>
       </x:c>
-      <x:c r="Y5" s="35" t="str">
+      <x:c r="Y5" s="36" t="str">
         <x:v>Score</x:v>
       </x:c>
-      <x:c r="Z5" s="35" t="str">
+      <x:c r="Z5" s="36" t="str">
         <x:v>Rate</x:v>
       </x:c>
-      <x:c r="AA5" s="35" t="str">
+      <x:c r="AA5" s="36" t="str">
         <x:v>Score</x:v>
       </x:c>
-      <x:c r="AB5" s="35" t="str">
+      <x:c r="AB5" s="36" t="str">
         <x:v>Rate</x:v>
       </x:c>
-      <x:c r="AC5" s="35" t="str">
+      <x:c r="AC5" s="36" t="str">
         <x:v>Score</x:v>
       </x:c>
-      <x:c r="AD5" s="35" t="str">
+      <x:c r="AD5" s="36" t="str">
         <x:v>Rate</x:v>
       </x:c>
-      <x:c r="AE5" s="35" t="str">
+      <x:c r="AE5" s="36" t="str">
         <x:v>Score</x:v>
       </x:c>
-      <x:c r="AF5" s="35" t="str">
+      <x:c r="AF5" s="36" t="str">
         <x:v>Rate</x:v>
       </x:c>
-      <x:c r="AG5" s="35" t="str">
+      <x:c r="AG5" s="36" t="str">
         <x:v>Score</x:v>
       </x:c>
-      <x:c r="AH5" s="35" t="str">
+      <x:c r="AH5" s="36" t="str">
         <x:v>Rate</x:v>
       </x:c>
-      <x:c r="AI5" s="35" t="str">
+      <x:c r="AI5" s="36" t="str">
         <x:v>Score</x:v>
       </x:c>
-      <x:c r="AJ5" s="35" t="str">
+      <x:c r="AJ5" s="36" t="str">
         <x:v>Rate</x:v>
       </x:c>
-      <x:c r="AK5" s="35" t="str">
+      <x:c r="AK5" s="36" t="str">
         <x:v>Score</x:v>
       </x:c>
-      <x:c r="AL5" s="35" t="str">
+      <x:c r="AL5" s="36" t="str">
         <x:v>Rate</x:v>
       </x:c>
-      <x:c r="AM5" s="35" t="str">
+      <x:c r="AM5" s="36" t="str">
         <x:v>Score</x:v>
       </x:c>
-      <x:c r="AN5" s="35" t="str">
+      <x:c r="AN5" s="36" t="str">
         <x:v>Rate</x:v>
       </x:c>
-      <x:c r="AO5" s="35" t="str">
+      <x:c r="AO5" s="36" t="str">
         <x:v>Score</x:v>
       </x:c>
-      <x:c r="AP5" s="35" t="str">
+      <x:c r="AP5" s="36" t="str">
         <x:v>Rate</x:v>
       </x:c>
       <x:c r="AQ5" s="13" t="str">
@@ -2231,10 +2231,10 @@
         <x:v>Supply crossing</x:v>
       </x:c>
       <x:c r="AU5" s="13" t="str">
-        <x:v>Velocity</x:v>
+        <x:v>First projected growth</x:v>
       </x:c>
       <x:c r="AV5" s="13" t="str">
-        <x:v>Acceleration</x:v>
+        <x:v>Pipeline acceleration</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" hidden="0" customHeight="1">
@@ -2244,170 +2244,170 @@
       <x:c r="B6" s="17" t="str">
         <x:v>Supported high-autonomy users ÷ 50% of U.S. resident population; capped at 100%</x:v>
       </x:c>
-      <x:c r="C6" s="45" t="n">
+      <x:c r="C6" s="46" t="n">
         <x:f>'Quarterly Model'!J6</x:f>
         <x:v>0.00682782226716592</x:v>
       </x:c>
-      <x:c r="D6" s="45" t="str">
+      <x:c r="D6" s="46" t="str">
         <x:f>'Quarterly Model'!K6</x:f>
       </x:c>
-      <x:c r="E6" s="45" t="n">
+      <x:c r="E6" s="46" t="n">
         <x:f>'Quarterly Model'!J7</x:f>
         <x:v>0.01320844974682248</x:v>
       </x:c>
-      <x:c r="F6" s="45" t="n">
+      <x:c r="F6" s="46" t="n">
         <x:f>'Quarterly Model'!K7</x:f>
         <x:v>0.006380627479656559</x:v>
       </x:c>
-      <x:c r="G6" s="45" t="n">
+      <x:c r="G6" s="46" t="n">
         <x:f>'Quarterly Model'!J8</x:f>
         <x:v>0.020071791898291506</x:v>
       </x:c>
-      <x:c r="H6" s="45" t="n">
+      <x:c r="H6" s="46" t="n">
         <x:f>'Quarterly Model'!K8</x:f>
         <x:v>0.006863342151469026</x:v>
       </x:c>
-      <x:c r="I6" s="45" t="n">
+      <x:c r="I6" s="46" t="n">
         <x:f>'Quarterly Model'!J9</x:f>
         <x:v>0.02814028092242638</x:v>
       </x:c>
-      <x:c r="J6" s="45" t="n">
+      <x:c r="J6" s="46" t="n">
         <x:f>'Quarterly Model'!K9</x:f>
         <x:v>0.008068489024134873</x:v>
       </x:c>
-      <x:c r="K6" s="45" t="n">
+      <x:c r="K6" s="46" t="n">
         <x:f>'Quarterly Model'!J10</x:f>
         <x:v>0.037555468283042195</x:v>
       </x:c>
-      <x:c r="L6" s="45" t="n">
+      <x:c r="L6" s="46" t="n">
         <x:f>'Quarterly Model'!K10</x:f>
         <x:v>0.009415187360615817</x:v>
       </x:c>
-      <x:c r="M6" s="45" t="n">
+      <x:c r="M6" s="46" t="n">
         <x:f>'Quarterly Model'!J11</x:f>
         <x:v>0.06633924833009283</x:v>
       </x:c>
-      <x:c r="N6" s="45" t="n">
+      <x:c r="N6" s="46" t="n">
         <x:f>'Quarterly Model'!K11</x:f>
         <x:v>0.028783780047050636</x:v>
       </x:c>
-      <x:c r="O6" s="45" t="n">
+      <x:c r="O6" s="46" t="n">
         <x:f>'Quarterly Model'!J12</x:f>
         <x:v>0.08726162750476324</x:v>
       </x:c>
-      <x:c r="P6" s="45" t="n">
+      <x:c r="P6" s="46" t="n">
         <x:f>'Quarterly Model'!K12</x:f>
         <x:v>0.020922379174670408</x:v>
       </x:c>
-      <x:c r="Q6" s="45" t="n">
+      <x:c r="Q6" s="46" t="n">
         <x:f>'Quarterly Model'!J13</x:f>
         <x:v>0.14706496698305438</x:v>
       </x:c>
-      <x:c r="R6" s="45" t="n">
+      <x:c r="R6" s="46" t="n">
         <x:f>'Quarterly Model'!K13</x:f>
         <x:v>0.05980333947829114</x:v>
       </x:c>
-      <x:c r="S6" s="45" t="n">
+      <x:c r="S6" s="46" t="n">
         <x:f>'Quarterly Model'!J14</x:f>
         <x:v>0.17513398579018094</x:v>
       </x:c>
-      <x:c r="T6" s="45" t="n">
+      <x:c r="T6" s="46" t="n">
         <x:f>'Quarterly Model'!K14</x:f>
         <x:v>0.02806901880712656</x:v>
       </x:c>
-      <x:c r="U6" s="45" t="n">
+      <x:c r="U6" s="46" t="n">
         <x:f>'Quarterly Model'!J15</x:f>
         <x:v>0.31194838109141576</x:v>
       </x:c>
-      <x:c r="V6" s="45" t="n">
+      <x:c r="V6" s="46" t="n">
         <x:f>'Quarterly Model'!K15</x:f>
         <x:v>0.13681439530123482</x:v>
       </x:c>
-      <x:c r="W6" s="45" t="n">
+      <x:c r="W6" s="46" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
         <x:v>0.37587725229616675</x:v>
       </x:c>
-      <x:c r="X6" s="45" t="n">
+      <x:c r="X6" s="46" t="n">
         <x:f>'Quarterly Model'!K16</x:f>
         <x:v>0.06392887120475099</x:v>
       </x:c>
-      <x:c r="Y6" s="33" t="n">
+      <x:c r="Y6" s="34" t="n">
         <x:f>'Quarterly Model'!J17</x:f>
-        <x:v>0.5038169880198742</x:v>
-      </x:c>
-      <x:c r="Z6" s="33" t="n">
+        <x:v>0.48359766611943783</x:v>
+      </x:c>
+      <x:c r="Z6" s="34" t="n">
         <x:f>'Quarterly Model'!K17</x:f>
-        <x:v>0.12793973572370743</x:v>
-      </x:c>
-      <x:c r="AA6" s="33" t="n">
+        <x:v>0.10772041382327108</x:v>
+      </x:c>
+      <x:c r="AA6" s="34" t="n">
         <x:f>'Quarterly Model'!J18</x:f>
-        <x:v>0.660890709854224</x:v>
-      </x:c>
-      <x:c r="AB6" s="33" t="n">
+        <x:v>0.5660964606872011</x:v>
+      </x:c>
+      <x:c r="AB6" s="34" t="n">
         <x:f>'Quarterly Model'!K18</x:f>
-        <x:v>0.15707372183434987</x:v>
-      </x:c>
-      <x:c r="AC6" s="33" t="n">
+        <x:v>0.08249879456776327</x:v>
+      </x:c>
+      <x:c r="AC6" s="34" t="n">
         <x:f>'Quarterly Model'!J19</x:f>
-        <x:v>0.8484310673527545</x:v>
-      </x:c>
-      <x:c r="AD6" s="33" t="n">
+        <x:v>0.5958694611740921</x:v>
+      </x:c>
+      <x:c r="AD6" s="34" t="n">
         <x:f>'Quarterly Model'!K19</x:f>
-        <x:v>0.18754035749853049</x:v>
-      </x:c>
-      <x:c r="AE6" s="33" t="n">
+        <x:v>0.02977300048689102</x:v>
+      </x:c>
+      <x:c r="AE6" s="34" t="n">
         <x:f>'Quarterly Model'!J20</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AF6" s="33" t="n">
+        <x:v>0.6459829039518208</x:v>
+      </x:c>
+      <x:c r="AF6" s="34" t="n">
         <x:f>'Quarterly Model'!K20</x:f>
-        <x:v>0.15156893264724547</x:v>
-      </x:c>
-      <x:c r="AG6" s="33" t="n">
+        <x:v>0.05011344277772867</x:v>
+      </x:c>
+      <x:c r="AG6" s="34" t="n">
         <x:f>'Quarterly Model'!J21</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AH6" s="33" t="n">
+        <x:v>0.8354035263994427</x:v>
+      </x:c>
+      <x:c r="AH6" s="34" t="n">
         <x:f>'Quarterly Model'!K21</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AI6" s="33" t="n">
+        <x:v>0.18942062244762192</x:v>
+      </x:c>
+      <x:c r="AI6" s="34" t="n">
         <x:f>'Quarterly Model'!J22</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AJ6" s="33" t="n">
+      <x:c r="AJ6" s="34" t="n">
         <x:f>'Quarterly Model'!K22</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AK6" s="33" t="n">
+        <x:v>0.1645964736005573</x:v>
+      </x:c>
+      <x:c r="AK6" s="34" t="n">
         <x:f>'Quarterly Model'!J23</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AL6" s="33" t="n">
+      <x:c r="AL6" s="34" t="n">
         <x:f>'Quarterly Model'!K23</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="AM6" s="33" t="n">
+      <x:c r="AM6" s="34" t="n">
         <x:f>'Quarterly Model'!J24</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AN6" s="33" t="n">
+      <x:c r="AN6" s="34" t="n">
         <x:f>'Quarterly Model'!K24</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="AO6" s="33" t="n">
+      <x:c r="AO6" s="34" t="n">
         <x:f>'Quarterly Model'!J25</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AP6" s="33" t="n">
+      <x:c r="AP6" s="34" t="n">
         <x:f>'Quarterly Model'!K25</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="AQ6" s="29" t="n">
+      <x:c r="AQ6" s="31" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
         <x:v>0.37587725229616675</x:v>
       </x:c>
-      <x:c r="AR6" s="29" t="str">
+      <x:c r="AR6" s="31" t="str">
         <x:f>'Quarterly Model'!L16</x:f>
         <x:v>F</x:v>
       </x:c>
@@ -2417,15 +2417,15 @@
       </x:c>
       <x:c r="AT6" s="20" t="n">
         <x:f>'Assumptions'!B32</x:f>
-        <x:v>46632.108708204854</x:v>
+        <x:v>46829.09207929863</x:v>
       </x:c>
       <x:c r="AU6" s="27" t="n">
         <x:f>'Assumptions'!B30</x:f>
-        <x:v>0.4382012678196282</x:v>
+        <x:v>0.3635456744374075</x:v>
       </x:c>
       <x:c r="AV6" s="27" t="n">
         <x:f>'Assumptions'!B28</x:f>
-        <x:v>-0.03112621365907439</x:v>
+        <x:v>0.003372652996279868</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2568,43 +2568,43 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
       <x:c r="I3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
       <x:c r="L3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
       <x:c r="M3" s="6" t="str">
-        <x:v>Observed capacity through 2026-Q3; later quarters extrapolate the smoothed quarterly log-growth velocity and acceleration. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
+        <x:v>Observed capacity through 2026-Q3; later quarters aggregate the expected/projected site states in Epoch's dated buildout pipeline. Score is supported users ÷ 50% U.S. population, capped at 100%.</x:v>
       </x:c>
     </x:row>
     <x:row r="4"/>
@@ -2663,7 +2663,7 @@
         <x:v>Observed</x:v>
       </x:c>
       <x:c r="E6" s="18" t="n">
-        <x:f>SUMIFS('Observations'!$D$6:$D$16,'Observations'!$A$6:$A$16,A6)</x:f>
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A6)</x:f>
         <x:v>245664</x:v>
       </x:c>
       <x:c r="F6" s="27" t="n">
@@ -2673,19 +2673,19 @@
       <x:c r="G6" s="27" t="str">
         <x:f>""</x:f>
       </x:c>
-      <x:c r="H6" s="28" t="n">
-        <x:f>E6*'Assumptions'!$B$24</x:f>
+      <x:c r="H6" s="30" t="n">
+        <x:f>E6*'Assumptions'!$B$25</x:f>
         <x:v>19602336337920</x:v>
       </x:c>
       <x:c r="I6" s="18" t="n">
         <x:f>H6/'Assumptions'!$I$11</x:f>
         <x:v>1170288.7365922388</x:v>
       </x:c>
-      <x:c r="J6" s="29" t="n">
+      <x:c r="J6" s="31" t="n">
         <x:f>MIN(1,I6/'Assumptions'!$B$9)</x:f>
         <x:v>0.00682782226716592</x:v>
       </x:c>
-      <x:c r="K6" s="29" t="str">
+      <x:c r="K6" s="31" t="str">
         <x:f>""</x:f>
       </x:c>
       <x:c r="L6" s="17" t="str">
@@ -2711,7 +2711,7 @@
         <x:v>Observed</x:v>
       </x:c>
       <x:c r="E7" s="18" t="n">
-        <x:f>SUMIFS('Observations'!$D$6:$D$16,'Observations'!$A$6:$A$16,A7)</x:f>
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A7)</x:f>
         <x:v>475238</x:v>
       </x:c>
       <x:c r="F7" s="27" t="n">
@@ -2722,19 +2722,19 @@
         <x:f>F7-F6</x:f>
         <x:v>0.9519637402300738</x:v>
       </x:c>
-      <x:c r="H7" s="28" t="n">
-        <x:f>E7*'Assumptions'!$B$24</x:f>
+      <x:c r="H7" s="30" t="n">
+        <x:f>E7*'Assumptions'!$B$25</x:f>
         <x:v>37920798800640</x:v>
       </x:c>
       <x:c r="I7" s="18" t="n">
         <x:f>H7/'Assumptions'!$I$11</x:f>
         <x:v>2263928.286605373</x:v>
       </x:c>
-      <x:c r="J7" s="29" t="n">
+      <x:c r="J7" s="31" t="n">
         <x:f>MIN(1,I7/'Assumptions'!$B$9)</x:f>
         <x:v>0.01320844974682248</x:v>
       </x:c>
-      <x:c r="K7" s="29" t="n">
+      <x:c r="K7" s="31" t="n">
         <x:f>J7-J6</x:f>
         <x:v>0.006380627479656559</x:v>
       </x:c>
@@ -2761,7 +2761,7 @@
         <x:v>Observed</x:v>
       </x:c>
       <x:c r="E8" s="18" t="n">
-        <x:f>SUMIFS('Observations'!$D$6:$D$16,'Observations'!$A$6:$A$16,A8)</x:f>
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A8)</x:f>
         <x:v>722180</x:v>
       </x:c>
       <x:c r="F8" s="27" t="n">
@@ -2772,19 +2772,19 @@
         <x:f>F8-F7</x:f>
         <x:v>0.6037082683951738</x:v>
       </x:c>
-      <x:c r="H8" s="28" t="n">
-        <x:f>E8*'Assumptions'!$B$24</x:f>
+      <x:c r="H8" s="30" t="n">
+        <x:f>E8*'Assumptions'!$B$25</x:f>
         <x:v>57625110950400</x:v>
       </x:c>
       <x:c r="I8" s="18" t="n">
         <x:f>H8/'Assumptions'!$I$11</x:f>
         <x:v>3440305.131367164</x:v>
       </x:c>
-      <x:c r="J8" s="29" t="n">
+      <x:c r="J8" s="31" t="n">
         <x:f>MIN(1,I8/'Assumptions'!$B$9)</x:f>
         <x:v>0.020071791898291506</x:v>
       </x:c>
-      <x:c r="K8" s="29" t="n">
+      <x:c r="K8" s="31" t="n">
         <x:f>J8-J7</x:f>
         <x:v>0.006863342151469026</x:v>
       </x:c>
@@ -2811,7 +2811,7 @@
         <x:v>Observed</x:v>
       </x:c>
       <x:c r="E9" s="18" t="n">
-        <x:f>SUMIFS('Observations'!$D$6:$D$16,'Observations'!$A$6:$A$16,A9)</x:f>
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A9)</x:f>
         <x:v>1012483</x:v>
       </x:c>
       <x:c r="F9" s="27" t="n">
@@ -2822,19 +2822,19 @@
         <x:f>F9-F8</x:f>
         <x:v>0.48746731270438204</x:v>
       </x:c>
-      <x:c r="H9" s="28" t="n">
-        <x:f>E9*'Assumptions'!$B$24</x:f>
+      <x:c r="H9" s="30" t="n">
+        <x:f>E9*'Assumptions'!$B$25</x:f>
         <x:v>80789339514240</x:v>
       </x:c>
       <x:c r="I9" s="18" t="n">
         <x:f>H9/'Assumptions'!$I$11</x:f>
         <x:v>4823244.150103881</x:v>
       </x:c>
-      <x:c r="J9" s="29" t="n">
+      <x:c r="J9" s="31" t="n">
         <x:f>MIN(1,I9/'Assumptions'!$B$9)</x:f>
         <x:v>0.02814028092242638</x:v>
       </x:c>
-      <x:c r="K9" s="29" t="n">
+      <x:c r="K9" s="31" t="n">
         <x:f>J9-J8</x:f>
         <x:v>0.008068489024134873</x:v>
       </x:c>
@@ -2861,7 +2861,7 @@
         <x:v>Observed</x:v>
       </x:c>
       <x:c r="E10" s="18" t="n">
-        <x:f>SUMIFS('Observations'!$D$6:$D$16,'Observations'!$A$6:$A$16,A10)</x:f>
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A10)</x:f>
         <x:v>1351240</x:v>
       </x:c>
       <x:c r="F10" s="27" t="n">
@@ -2872,19 +2872,19 @@
         <x:f>F10-F9</x:f>
         <x:v>0.416386256410302</x:v>
       </x:c>
-      <x:c r="H10" s="28" t="n">
-        <x:f>E10*'Assumptions'!$B$24</x:f>
+      <x:c r="H10" s="30" t="n">
+        <x:f>E10*'Assumptions'!$B$25</x:f>
         <x:v>107819871667200</x:v>
       </x:c>
       <x:c r="I10" s="18" t="n">
         <x:f>H10/'Assumptions'!$I$11</x:f>
         <x:v>6437007.2637134325</x:v>
       </x:c>
-      <x:c r="J10" s="29" t="n">
+      <x:c r="J10" s="31" t="n">
         <x:f>MIN(1,I10/'Assumptions'!$B$9)</x:f>
         <x:v>0.037555468283042195</x:v>
       </x:c>
-      <x:c r="K10" s="29" t="n">
+      <x:c r="K10" s="31" t="n">
         <x:f>J10-J9</x:f>
         <x:v>0.009415187360615817</x:v>
       </x:c>
@@ -2911,7 +2911,7 @@
         <x:v>Observed</x:v>
       </x:c>
       <x:c r="E11" s="18" t="n">
-        <x:f>SUMIFS('Observations'!$D$6:$D$16,'Observations'!$A$6:$A$16,A11)</x:f>
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A11)</x:f>
         <x:v>2386876</x:v>
       </x:c>
       <x:c r="F11" s="27" t="n">
@@ -2922,19 +2922,19 @@
         <x:f>F11-F10</x:f>
         <x:v>0.8208396780997056</x:v>
       </x:c>
-      <x:c r="H11" s="28" t="n">
-        <x:f>E11*'Assumptions'!$B$24</x:f>
+      <x:c r="H11" s="30" t="n">
+        <x:f>E11*'Assumptions'!$B$25</x:f>
         <x:v>190456664993280</x:v>
       </x:c>
       <x:c r="I11" s="18" t="n">
         <x:f>H11/'Assumptions'!$I$11</x:f>
         <x:v>11370547.16377791</x:v>
       </x:c>
-      <x:c r="J11" s="29" t="n">
+      <x:c r="J11" s="31" t="n">
         <x:f>MIN(1,I11/'Assumptions'!$B$9)</x:f>
         <x:v>0.06633924833009283</x:v>
       </x:c>
-      <x:c r="K11" s="29" t="n">
+      <x:c r="K11" s="31" t="n">
         <x:f>J11-J10</x:f>
         <x:v>0.028783780047050636</x:v>
       </x:c>
@@ -2961,7 +2961,7 @@
         <x:v>Observed</x:v>
       </x:c>
       <x:c r="E12" s="18" t="n">
-        <x:f>SUMIFS('Observations'!$D$6:$D$16,'Observations'!$A$6:$A$16,A12)</x:f>
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A12)</x:f>
         <x:v>3139660</x:v>
       </x:c>
       <x:c r="F12" s="27" t="n">
@@ -2972,19 +2972,19 @@
         <x:f>F12-F11</x:f>
         <x:v>0.3954847159961119</x:v>
       </x:c>
-      <x:c r="H12" s="28" t="n">
-        <x:f>E12*'Assumptions'!$B$24</x:f>
+      <x:c r="H12" s="30" t="n">
+        <x:f>E12*'Assumptions'!$B$25</x:f>
         <x:v>250523769484800</x:v>
       </x:c>
       <x:c r="I12" s="18" t="n">
         <x:f>H12/'Assumptions'!$I$11</x:f>
         <x:v>14956642.954316419</x:v>
       </x:c>
-      <x:c r="J12" s="29" t="n">
+      <x:c r="J12" s="31" t="n">
         <x:f>MIN(1,I12/'Assumptions'!$B$9)</x:f>
         <x:v>0.08726162750476324</x:v>
       </x:c>
-      <x:c r="K12" s="29" t="n">
+      <x:c r="K12" s="31" t="n">
         <x:f>J12-J11</x:f>
         <x:v>0.020922379174670408</x:v>
       </x:c>
@@ -3011,7 +3011,7 @@
         <x:v>Observed</x:v>
       </x:c>
       <x:c r="E13" s="18" t="n">
-        <x:f>SUMIFS('Observations'!$D$6:$D$16,'Observations'!$A$6:$A$16,A13)</x:f>
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A13)</x:f>
         <x:v>5291375</x:v>
       </x:c>
       <x:c r="F13" s="27" t="n">
@@ -3022,19 +3022,19 @@
         <x:f>F13-F12</x:f>
         <x:v>0.7530343299629934</x:v>
       </x:c>
-      <x:c r="H13" s="28" t="n">
-        <x:f>E13*'Assumptions'!$B$24</x:f>
+      <x:c r="H13" s="30" t="n">
+        <x:f>E13*'Assumptions'!$B$25</x:f>
         <x:v>422216166960000</x:v>
       </x:c>
       <x:c r="I13" s="18" t="n">
         <x:f>H13/'Assumptions'!$I$11</x:f>
         <x:v>25206935.340895522</x:v>
       </x:c>
-      <x:c r="J13" s="29" t="n">
+      <x:c r="J13" s="31" t="n">
         <x:f>MIN(1,I13/'Assumptions'!$B$9)</x:f>
         <x:v>0.14706496698305438</x:v>
       </x:c>
-      <x:c r="K13" s="29" t="n">
+      <x:c r="K13" s="31" t="n">
         <x:f>J13-J12</x:f>
         <x:v>0.05980333947829114</x:v>
       </x:c>
@@ -3061,7 +3061,7 @@
         <x:v>Observed</x:v>
       </x:c>
       <x:c r="E14" s="18" t="n">
-        <x:f>SUMIFS('Observations'!$D$6:$D$16,'Observations'!$A$6:$A$16,A14)</x:f>
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A14)</x:f>
         <x:v>6301294</x:v>
       </x:c>
       <x:c r="F14" s="27" t="n">
@@ -3072,19 +3072,19 @@
         <x:f>F14-F13</x:f>
         <x:v>0.2520054579308564</x:v>
       </x:c>
-      <x:c r="H14" s="28" t="n">
-        <x:f>E14*'Assumptions'!$B$24</x:f>
+      <x:c r="H14" s="30" t="n">
+        <x:f>E14*'Assumptions'!$B$25</x:f>
         <x:v>502800916504320</x:v>
       </x:c>
       <x:c r="I14" s="18" t="n">
         <x:f>H14/'Assumptions'!$I$11</x:f>
         <x:v>30017965.164437015</x:v>
       </x:c>
-      <x:c r="J14" s="29" t="n">
+      <x:c r="J14" s="31" t="n">
         <x:f>MIN(1,I14/'Assumptions'!$B$9)</x:f>
         <x:v>0.17513398579018094</x:v>
       </x:c>
-      <x:c r="K14" s="29" t="n">
+      <x:c r="K14" s="31" t="n">
         <x:f>J14-J13</x:f>
         <x:v>0.02806901880712656</x:v>
       </x:c>
@@ -3111,7 +3111,7 @@
         <x:v>Observed</x:v>
       </x:c>
       <x:c r="E15" s="18" t="n">
-        <x:f>SUMIFS('Observations'!$D$6:$D$16,'Observations'!$A$6:$A$16,A15)</x:f>
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A15)</x:f>
         <x:v>11223855</x:v>
       </x:c>
       <x:c r="F15" s="27" t="n">
@@ -3122,19 +3122,19 @@
         <x:f>F15-F14</x:f>
         <x:v>0.8328482478612642</x:v>
       </x:c>
-      <x:c r="H15" s="28" t="n">
-        <x:f>E15*'Assumptions'!$B$24</x:f>
+      <x:c r="H15" s="30" t="n">
+        <x:f>E15*'Assumptions'!$B$25</x:f>
         <x:v>895588204694400</x:v>
       </x:c>
       <x:c r="I15" s="18" t="n">
         <x:f>H15/'Assumptions'!$I$11</x:f>
         <x:v>53467952.51906866</x:v>
       </x:c>
-      <x:c r="J15" s="29" t="n">
+      <x:c r="J15" s="31" t="n">
         <x:f>MIN(1,I15/'Assumptions'!$B$9)</x:f>
         <x:v>0.31194838109141576</x:v>
       </x:c>
-      <x:c r="K15" s="29" t="n">
+      <x:c r="K15" s="31" t="n">
         <x:f>J15-J14</x:f>
         <x:v>0.13681439530123482</x:v>
       </x:c>
@@ -3161,7 +3161,7 @@
         <x:v>Observed QTD</x:v>
       </x:c>
       <x:c r="E16" s="18" t="n">
-        <x:f>SUMIFS('Observations'!$D$6:$D$16,'Observations'!$A$6:$A$16,A16)</x:f>
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A16)</x:f>
         <x:v>13524006</x:v>
       </x:c>
       <x:c r="F16" s="27" t="n">
@@ -3172,19 +3172,19 @@
         <x:f>F16-F15</x:f>
         <x:v>0.2689542852637672</x:v>
       </x:c>
-      <x:c r="H16" s="28" t="n">
-        <x:f>E16*'Assumptions'!$B$24</x:f>
+      <x:c r="H16" s="30" t="n">
+        <x:f>E16*'Assumptions'!$B$25</x:f>
         <x:v>1079124797479680</x:v>
       </x:c>
       <x:c r="I16" s="18" t="n">
         <x:f>H16/'Assumptions'!$I$11</x:f>
         <x:v>64425361.043562986</x:v>
       </x:c>
-      <x:c r="J16" s="29" t="n">
+      <x:c r="J16" s="31" t="n">
         <x:f>MIN(1,I16/'Assumptions'!$B$9)</x:f>
         <x:v>0.37587725229616675</x:v>
       </x:c>
-      <x:c r="K16" s="29" t="n">
+      <x:c r="K16" s="31" t="n">
         <x:f>J16-J15</x:f>
         <x:v>0.06392887120475099</x:v>
       </x:c>
@@ -3210,39 +3210,39 @@
       <x:c r="D17" s="23" t="str">
         <x:v>Projected</x:v>
       </x:c>
-      <x:c r="E17" s="30" t="n">
-        <x:f>POWER(2,MAX($F$16,$F$16+'Assumptions'!$B$30*(A17-'Assumptions'!$B$10)+0.5*'Assumptions'!$B$28*POWER(A17-'Assumptions'!$B$10,2)))</x:f>
-        <x:v>18127258.106893934</x:v>
-      </x:c>
-      <x:c r="F17" s="31" t="n">
+      <x:c r="E17" s="29" t="n">
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A17)</x:f>
+        <x:v>17399770</x:v>
+      </x:c>
+      <x:c r="F17" s="32" t="n">
         <x:f>LN(E17)/LN(2)</x:f>
-        <x:v>24.11165738660533</x:v>
-      </x:c>
-      <x:c r="G17" s="31" t="n">
+        <x:v>24.05256490005264</x:v>
+      </x:c>
+      <x:c r="G17" s="32" t="n">
         <x:f>F17-F16</x:f>
-        <x:v>0.4226381609900969</x:v>
-      </x:c>
-      <x:c r="H17" s="32" t="n">
-        <x:f>E17*'Assumptions'!$B$24</x:f>
-        <x:v>1446433381755657.8</x:v>
-      </x:c>
-      <x:c r="I17" s="30" t="n">
+        <x:v>0.3635456744374075</x:v>
+      </x:c>
+      <x:c r="H17" s="33" t="n">
+        <x:f>E17*'Assumptions'!$B$25</x:f>
+        <x:v>1388384719545600</x:v>
+      </x:c>
+      <x:c r="I17" s="29" t="n">
         <x:f>H17/'Assumptions'!$I$11</x:f>
-        <x:v>86354231.74660644</x:v>
-      </x:c>
-      <x:c r="J17" s="33" t="n">
+        <x:v>82888639.97287165</x:v>
+      </x:c>
+      <x:c r="J17" s="34" t="n">
         <x:f>MIN(1,I17/'Assumptions'!$B$9)</x:f>
-        <x:v>0.5038169880198742</x:v>
-      </x:c>
-      <x:c r="K17" s="33" t="n">
+        <x:v>0.48359766611943783</x:v>
+      </x:c>
+      <x:c r="K17" s="34" t="n">
         <x:f>J17-J16</x:f>
-        <x:v>0.12793973572370743</x:v>
+        <x:v>0.10772041382327108</x:v>
       </x:c>
       <x:c r="L17" s="23" t="str">
         <x:f>IF(J17&gt;='Assumptions'!$G$16,"A",IF(J17&gt;='Assumptions'!$G$17,"B",IF(J17&gt;='Assumptions'!$G$18,"C",IF(J17&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
         <x:v>F</x:v>
       </x:c>
-      <x:c r="M17" s="34" t="n">
+      <x:c r="M17" s="35" t="n">
         <x:f>IF(J17&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J17&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J17&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J17&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -3260,41 +3260,41 @@
       <x:c r="D18" s="23" t="str">
         <x:v>Projected</x:v>
       </x:c>
-      <x:c r="E18" s="30" t="n">
-        <x:f>POWER(2,MAX($F$16,$F$16+'Assumptions'!$B$30*(A18-'Assumptions'!$B$10)+0.5*'Assumptions'!$B$28*POWER(A18-'Assumptions'!$B$10,2)))</x:f>
-        <x:v>23778746.574347917</x:v>
-      </x:c>
-      <x:c r="F18" s="31" t="n">
+      <x:c r="E18" s="29" t="n">
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A18)</x:f>
+        <x:v>20368064</x:v>
+      </x:c>
+      <x:c r="F18" s="32" t="n">
         <x:f>LN(E18)/LN(2)</x:f>
-        <x:v>24.50316933393634</x:v>
-      </x:c>
-      <x:c r="G18" s="31" t="n">
+        <x:v>24.279805521769333</x:v>
+      </x:c>
+      <x:c r="G18" s="32" t="n">
         <x:f>F18-F17</x:f>
-        <x:v>0.39151194733101136</x:v>
-      </x:c>
-      <x:c r="H18" s="32" t="n">
-        <x:f>E18*'Assumptions'!$B$24</x:f>
-        <x:v>1897384183455984.2</x:v>
-      </x:c>
-      <x:c r="I18" s="30" t="n">
+        <x:v>0.22724062171669246</x:v>
+      </x:c>
+      <x:c r="H18" s="33" t="n">
+        <x:f>E18*'Assumptions'!$B$25</x:f>
+        <x:v>1625234633809920</x:v>
+      </x:c>
+      <x:c r="I18" s="29" t="n">
         <x:f>H18/'Assumptions'!$I$11</x:f>
-        <x:v>113276667.66901399</x:v>
-      </x:c>
-      <x:c r="J18" s="33" t="n">
+        <x:v>97028933.36178628</x:v>
+      </x:c>
+      <x:c r="J18" s="34" t="n">
         <x:f>MIN(1,I18/'Assumptions'!$B$9)</x:f>
-        <x:v>0.660890709854224</x:v>
-      </x:c>
-      <x:c r="K18" s="33" t="n">
+        <x:v>0.5660964606872011</x:v>
+      </x:c>
+      <x:c r="K18" s="34" t="n">
         <x:f>J18-J17</x:f>
-        <x:v>0.15707372183434987</x:v>
+        <x:v>0.08249879456776327</x:v>
       </x:c>
       <x:c r="L18" s="23" t="str">
         <x:f>IF(J18&gt;='Assumptions'!$G$16,"A",IF(J18&gt;='Assumptions'!$G$17,"B",IF(J18&gt;='Assumptions'!$G$18,"C",IF(J18&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
-        <x:v>D</x:v>
-      </x:c>
-      <x:c r="M18" s="34" t="n">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="M18" s="35" t="n">
         <x:f>IF(J18&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J18&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J18&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J18&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -3310,41 +3310,41 @@
       <x:c r="D19" s="23" t="str">
         <x:v>Projected</x:v>
       </x:c>
-      <x:c r="E19" s="30" t="n">
-        <x:f>POWER(2,MAX($F$16,$F$16+'Assumptions'!$B$30*(A19-'Assumptions'!$B$10)+0.5*'Assumptions'!$B$28*POWER(A19-'Assumptions'!$B$10,2)))</x:f>
-        <x:v>30526419.9293022</x:v>
-      </x:c>
-      <x:c r="F19" s="31" t="n">
+      <x:c r="E19" s="29" t="n">
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A19)</x:f>
+        <x:v>21439292</x:v>
+      </x:c>
+      <x:c r="F19" s="32" t="n">
         <x:f>LN(E19)/LN(2)</x:f>
-        <x:v>24.86355506760828</x:v>
-      </x:c>
-      <x:c r="G19" s="31" t="n">
+        <x:v>24.3537539279851</x:v>
+      </x:c>
+      <x:c r="G19" s="32" t="n">
         <x:f>F19-F18</x:f>
-        <x:v>0.36038573367194005</x:v>
-      </x:c>
-      <x:c r="H19" s="32" t="n">
-        <x:f>E19*'Assumptions'!$B$24</x:f>
-        <x:v>2435803172816390.5</x:v>
-      </x:c>
-      <x:c r="I19" s="30" t="n">
+        <x:v>0.07394840621576648</x:v>
+      </x:c>
+      <x:c r="H19" s="33" t="n">
+        <x:f>E19*'Assumptions'!$B$25</x:f>
+        <x:v>1710711429557760</x:v>
+      </x:c>
+      <x:c r="I19" s="29" t="n">
         <x:f>H19/'Assumptions'!$I$11</x:f>
-        <x:v>145421084.94426212</x:v>
-      </x:c>
-      <x:c r="J19" s="33" t="n">
+        <x:v>102132025.6452394</x:v>
+      </x:c>
+      <x:c r="J19" s="34" t="n">
         <x:f>MIN(1,I19/'Assumptions'!$B$9)</x:f>
-        <x:v>0.8484310673527545</x:v>
-      </x:c>
-      <x:c r="K19" s="33" t="n">
+        <x:v>0.5958694611740921</x:v>
+      </x:c>
+      <x:c r="K19" s="34" t="n">
         <x:f>J19-J18</x:f>
-        <x:v>0.18754035749853049</x:v>
+        <x:v>0.02977300048689102</x:v>
       </x:c>
       <x:c r="L19" s="23" t="str">
         <x:f>IF(J19&gt;='Assumptions'!$G$16,"A",IF(J19&gt;='Assumptions'!$G$17,"B",IF(J19&gt;='Assumptions'!$G$18,"C",IF(J19&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="M19" s="34" t="n">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="M19" s="35" t="n">
         <x:f>IF(J19&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J19&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J19&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J19&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -3360,41 +3360,41 @@
       <x:c r="D20" s="23" t="str">
         <x:v>Projected</x:v>
       </x:c>
-      <x:c r="E20" s="30" t="n">
-        <x:f>POWER(2,MAX($F$16,$F$16+'Assumptions'!$B$30*(A20-'Assumptions'!$B$10)+0.5*'Assumptions'!$B$28*POWER(A20-'Assumptions'!$B$10,2)))</x:f>
-        <x:v>38352428.24553096</x:v>
-      </x:c>
-      <x:c r="F20" s="31" t="n">
+      <x:c r="E20" s="29" t="n">
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A20)</x:f>
+        <x:v>23242366</x:v>
+      </x:c>
+      <x:c r="F20" s="32" t="n">
         <x:f>LN(E20)/LN(2)</x:f>
-        <x:v>25.19281458762115</x:v>
-      </x:c>
-      <x:c r="G20" s="31" t="n">
+        <x:v>24.47025360226221</x:v>
+      </x:c>
+      <x:c r="G20" s="32" t="n">
         <x:f>F20-F19</x:f>
-        <x:v>0.32925952001286873</x:v>
-      </x:c>
-      <x:c r="H20" s="32" t="n">
-        <x:f>E20*'Assumptions'!$B$24</x:f>
-        <x:v>3060266045675561</x:v>
-      </x:c>
-      <x:c r="I20" s="30" t="n">
+        <x:v>0.11649967427711161</x:v>
+      </x:c>
+      <x:c r="H20" s="33" t="n">
+        <x:f>E20*'Assumptions'!$B$25</x:f>
+        <x:v>1854584618100480</x:v>
+      </x:c>
+      <x:c r="I20" s="29" t="n">
         <x:f>H20/'Assumptions'!$I$11</x:f>
-        <x:v>182702450.4880932</x:v>
-      </x:c>
-      <x:c r="J20" s="33" t="n">
+        <x:v>110721469.73734209</x:v>
+      </x:c>
+      <x:c r="J20" s="34" t="n">
         <x:f>MIN(1,I20/'Assumptions'!$B$9)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K20" s="33" t="n">
+        <x:v>0.6459829039518208</x:v>
+      </x:c>
+      <x:c r="K20" s="34" t="n">
         <x:f>J20-J19</x:f>
-        <x:v>0.15156893264724547</x:v>
+        <x:v>0.05011344277772867</x:v>
       </x:c>
       <x:c r="L20" s="23" t="str">
         <x:f>IF(J20&gt;='Assumptions'!$G$16,"A",IF(J20&gt;='Assumptions'!$G$17,"B",IF(J20&gt;='Assumptions'!$G$18,"C",IF(J20&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="M20" s="34" t="n">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="M20" s="35" t="n">
         <x:f>IF(J20&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J20&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J20&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J20&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -3410,41 +3410,41 @@
       <x:c r="D21" s="23" t="str">
         <x:v>Projected</x:v>
       </x:c>
-      <x:c r="E21" s="30" t="n">
-        <x:f>POWER(2,MAX($F$16,$F$16+'Assumptions'!$B$30*(A21-'Assumptions'!$B$10)+0.5*'Assumptions'!$B$28*POWER(A21-'Assumptions'!$B$10,2)))</x:f>
-        <x:v>47156323.02513182</x:v>
-      </x:c>
-      <x:c r="F21" s="31" t="n">
+      <x:c r="E21" s="29" t="n">
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A21)</x:f>
+        <x:v>30057691</x:v>
+      </x:c>
+      <x:c r="F21" s="32" t="n">
         <x:f>LN(E21)/LN(2)</x:f>
-        <x:v>25.490947893974944</x:v>
-      </x:c>
-      <x:c r="G21" s="31" t="n">
+        <x:v>24.84123085141674</x:v>
+      </x:c>
+      <x:c r="G21" s="32" t="n">
         <x:f>F21-F20</x:f>
-        <x:v>0.29813330635379387</x:v>
-      </x:c>
-      <x:c r="H21" s="32" t="n">
-        <x:f>E21*'Assumptions'!$B$24</x:f>
-        <x:v>3762757686914790.5</x:v>
-      </x:c>
-      <x:c r="I21" s="30" t="n">
+        <x:v>0.370977249154528</x:v>
+      </x:c>
+      <x:c r="H21" s="33" t="n">
+        <x:f>E21*'Assumptions'!$B$25</x:f>
+        <x:v>2398401754116480</x:v>
+      </x:c>
+      <x:c r="I21" s="29" t="n">
         <x:f>H21/'Assumptions'!$I$11</x:f>
-        <x:v>224642249.9650621</x:v>
-      </x:c>
-      <x:c r="J21" s="33" t="n">
+        <x:v>143188164.42486447</x:v>
+      </x:c>
+      <x:c r="J21" s="34" t="n">
         <x:f>MIN(1,I21/'Assumptions'!$B$9)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K21" s="33" t="n">
+        <x:v>0.8354035263994427</x:v>
+      </x:c>
+      <x:c r="K21" s="34" t="n">
         <x:f>J21-J20</x:f>
-        <x:v>0</x:v>
+        <x:v>0.18942062244762192</x:v>
       </x:c>
       <x:c r="L21" s="23" t="str">
         <x:f>IF(J21&gt;='Assumptions'!$G$16,"A",IF(J21&gt;='Assumptions'!$G$17,"B",IF(J21&gt;='Assumptions'!$G$18,"C",IF(J21&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
-        <x:v>A</x:v>
-      </x:c>
-      <x:c r="M21" s="34" t="n">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="M21" s="35" t="n">
         <x:f>IF(J21&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J21&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J21&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J21&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -3460,39 +3460,39 @@
       <x:c r="D22" s="23" t="str">
         <x:v>Projected</x:v>
       </x:c>
-      <x:c r="E22" s="30" t="n">
-        <x:f>POWER(2,MAX($F$16,$F$16+'Assumptions'!$B$30*(A22-'Assumptions'!$B$10)+0.5*'Assumptions'!$B$28*POWER(A22-'Assumptions'!$B$10,2)))</x:f>
-        <x:v>56743625.158091314</x:v>
-      </x:c>
-      <x:c r="F22" s="31" t="n">
+      <x:c r="E22" s="29" t="n">
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A22)</x:f>
+        <x:v>37048243</x:v>
+      </x:c>
+      <x:c r="F22" s="32" t="n">
         <x:f>LN(E22)/LN(2)</x:f>
-        <x:v>25.757954986669667</x:v>
-      </x:c>
-      <x:c r="G22" s="31" t="n">
+        <x:v>25.142901789055948</x:v>
+      </x:c>
+      <x:c r="G22" s="32" t="n">
         <x:f>F22-F21</x:f>
-        <x:v>0.26700709269472256</x:v>
-      </x:c>
-      <x:c r="H22" s="32" t="n">
-        <x:f>E22*'Assumptions'!$B$24</x:f>
-        <x:v>4527759970454624</x:v>
-      </x:c>
-      <x:c r="I22" s="30" t="n">
+        <x:v>0.3016709376392086</x:v>
+      </x:c>
+      <x:c r="H22" s="33" t="n">
+        <x:f>E22*'Assumptions'!$B$25</x:f>
+        <x:v>2956200827207040</x:v>
+      </x:c>
+      <x:c r="I22" s="29" t="n">
         <x:f>H22/'Assumptions'!$I$11</x:f>
-        <x:v>270314028.08684325</x:v>
-      </x:c>
-      <x:c r="J22" s="33" t="n">
+        <x:v>176489601.6243009</x:v>
+      </x:c>
+      <x:c r="J22" s="34" t="n">
         <x:f>MIN(1,I22/'Assumptions'!$B$9)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K22" s="33" t="n">
+      <x:c r="K22" s="34" t="n">
         <x:f>J22-J21</x:f>
-        <x:v>0</x:v>
+        <x:v>0.1645964736005573</x:v>
       </x:c>
       <x:c r="L22" s="23" t="str">
         <x:f>IF(J22&gt;='Assumptions'!$G$16,"A",IF(J22&gt;='Assumptions'!$G$17,"B",IF(J22&gt;='Assumptions'!$G$18,"C",IF(J22&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
         <x:v>A</x:v>
       </x:c>
-      <x:c r="M22" s="34" t="n">
+      <x:c r="M22" s="35" t="n">
         <x:f>IF(J22&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J22&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J22&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J22&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
         <x:v>4</x:v>
       </x:c>
@@ -3510,31 +3510,31 @@
       <x:c r="D23" s="23" t="str">
         <x:v>Projected</x:v>
       </x:c>
-      <x:c r="E23" s="30" t="n">
-        <x:f>POWER(2,MAX($F$16,$F$16+'Assumptions'!$B$30*(A23-'Assumptions'!$B$10)+0.5*'Assumptions'!$B$28*POWER(A23-'Assumptions'!$B$10,2)))</x:f>
-        <x:v>66822742.84080343</x:v>
-      </x:c>
-      <x:c r="F23" s="31" t="n">
+      <x:c r="E23" s="29" t="n">
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A23)</x:f>
+        <x:v>46037632</x:v>
+      </x:c>
+      <x:c r="F23" s="32" t="n">
         <x:f>LN(E23)/LN(2)</x:f>
-        <x:v>25.993835865705307</x:v>
-      </x:c>
-      <x:c r="G23" s="31" t="n">
+        <x:v>25.456310292865954</x:v>
+      </x:c>
+      <x:c r="G23" s="32" t="n">
         <x:f>F23-F22</x:f>
-        <x:v>0.2358808790356406</x:v>
-      </x:c>
-      <x:c r="H23" s="32" t="n">
-        <x:f>E23*'Assumptions'!$B$24</x:f>
-        <x:v>5332005829864223</x:v>
-      </x:c>
-      <x:c r="I23" s="30" t="n">
+        <x:v>0.31340850381000607</x:v>
+      </x:c>
+      <x:c r="H23" s="33" t="n">
+        <x:f>E23*'Assumptions'!$B$25</x:f>
+        <x:v>3673493660712960</x:v>
+      </x:c>
+      <x:c r="I23" s="29" t="n">
         <x:f>H23/'Assumptions'!$I$11</x:f>
-        <x:v>318328706.2605506</x:v>
-      </x:c>
-      <x:c r="J23" s="33" t="n">
+        <x:v>219313054.37092298</x:v>
+      </x:c>
+      <x:c r="J23" s="34" t="n">
         <x:f>MIN(1,I23/'Assumptions'!$B$9)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K23" s="33" t="n">
+      <x:c r="K23" s="34" t="n">
         <x:f>J23-J22</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -3542,7 +3542,7 @@
         <x:f>IF(J23&gt;='Assumptions'!$G$16,"A",IF(J23&gt;='Assumptions'!$G$17,"B",IF(J23&gt;='Assumptions'!$G$18,"C",IF(J23&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
         <x:v>A</x:v>
       </x:c>
-      <x:c r="M23" s="34" t="n">
+      <x:c r="M23" s="35" t="n">
         <x:f>IF(J23&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J23&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J23&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J23&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
         <x:v>4</x:v>
       </x:c>
@@ -3560,31 +3560,31 @@
       <x:c r="D24" s="23" t="str">
         <x:v>Projected</x:v>
       </x:c>
-      <x:c r="E24" s="30" t="n">
-        <x:f>POWER(2,MAX($F$16,$F$16+'Assumptions'!$B$30*(A24-'Assumptions'!$B$10)+0.5*'Assumptions'!$B$28*POWER(A24-'Assumptions'!$B$10,2)))</x:f>
-        <x:v>77012565.99657708</x:v>
-      </x:c>
-      <x:c r="F24" s="31" t="n">
+      <x:c r="E24" s="29" t="n">
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A24)</x:f>
+        <x:v>47106859</x:v>
+      </x:c>
+      <x:c r="F24" s="32" t="n">
         <x:f>LN(E24)/LN(2)</x:f>
-        <x:v>26.198590531081877</x:v>
-      </x:c>
-      <x:c r="G24" s="31" t="n">
+        <x:v>25.489433803133178</x:v>
+      </x:c>
+      <x:c r="G24" s="32" t="n">
         <x:f>F24-F23</x:f>
-        <x:v>0.20475466537656928</x:v>
-      </x:c>
-      <x:c r="H24" s="32" t="n">
-        <x:f>E24*'Assumptions'!$B$24</x:f>
-        <x:v>6145085242083354</x:v>
-      </x:c>
-      <x:c r="I24" s="30" t="n">
+        <x:v>0.03312351026722382</x:v>
+      </x:c>
+      <x:c r="H24" s="33" t="n">
+        <x:f>E24*'Assumptions'!$B$25</x:f>
+        <x:v>3758810790107520</x:v>
+      </x:c>
+      <x:c r="I24" s="29" t="n">
         <x:f>H24/'Assumptions'!$I$11</x:f>
-        <x:v>366870760.72139424</x:v>
-      </x:c>
-      <x:c r="J24" s="33" t="n">
+        <x:v>224406614.33477733</x:v>
+      </x:c>
+      <x:c r="J24" s="34" t="n">
         <x:f>MIN(1,I24/'Assumptions'!$B$9)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K24" s="33" t="n">
+      <x:c r="K24" s="34" t="n">
         <x:f>J24-J23</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -3592,7 +3592,7 @@
         <x:f>IF(J24&gt;='Assumptions'!$G$16,"A",IF(J24&gt;='Assumptions'!$G$17,"B",IF(J24&gt;='Assumptions'!$G$18,"C",IF(J24&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
         <x:v>A</x:v>
       </x:c>
-      <x:c r="M24" s="34" t="n">
+      <x:c r="M24" s="35" t="n">
         <x:f>IF(J24&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J24&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J24&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J24&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
         <x:v>4</x:v>
       </x:c>
@@ -3610,31 +3610,31 @@
       <x:c r="D25" s="23" t="str">
         <x:v>Projected</x:v>
       </x:c>
-      <x:c r="E25" s="30" t="n">
-        <x:f>POWER(2,MAX($F$16,$F$16+'Assumptions'!$B$30*(A25-'Assumptions'!$B$10)+0.5*'Assumptions'!$B$28*POWER(A25-'Assumptions'!$B$10,2)))</x:f>
-        <x:v>86861828.24555889</x:v>
-      </x:c>
-      <x:c r="F25" s="31" t="n">
+      <x:c r="E25" s="29" t="n">
+        <x:f>SUMIFS('Observations'!$D$6:$D$25,'Observations'!$A$6:$A$25,A25)</x:f>
+        <x:v>61887051</x:v>
+      </x:c>
+      <x:c r="F25" s="32" t="n">
         <x:f>LN(E25)/LN(2)</x:f>
-        <x:v>26.372218982799378</x:v>
-      </x:c>
-      <x:c r="G25" s="31" t="n">
+        <x:v>25.88313424146424</x:v>
+      </x:c>
+      <x:c r="G25" s="32" t="n">
         <x:f>F25-F24</x:f>
-        <x:v>0.17362845171750152</x:v>
-      </x:c>
-      <x:c r="H25" s="32" t="n">
-        <x:f>E25*'Assumptions'!$B$24</x:f>
-        <x:v>6930990182509789</x:v>
-      </x:c>
-      <x:c r="I25" s="30" t="n">
+        <x:v>0.39370043833106294</x:v>
+      </x:c>
+      <x:c r="H25" s="33" t="n">
+        <x:f>E25*'Assumptions'!$B$25</x:f>
+        <x:v>4938170788817280</x:v>
+      </x:c>
+      <x:c r="I25" s="29" t="n">
         <x:f>H25/'Assumptions'!$I$11</x:f>
-        <x:v>413790458.65730083</x:v>
-      </x:c>
-      <x:c r="J25" s="33" t="n">
+        <x:v>294816166.496554</x:v>
+      </x:c>
+      <x:c r="J25" s="34" t="n">
         <x:f>MIN(1,I25/'Assumptions'!$B$9)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K25" s="33" t="n">
+      <x:c r="K25" s="34" t="n">
         <x:f>J25-J24</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -3642,7 +3642,7 @@
         <x:f>IF(J25&gt;='Assumptions'!$G$16,"A",IF(J25&gt;='Assumptions'!$G$17,"B",IF(J25&gt;='Assumptions'!$G$18,"C",IF(J25&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
         <x:v>A</x:v>
       </x:c>
-      <x:c r="M25" s="34" t="n">
+      <x:c r="M25" s="35" t="n">
         <x:f>IF(J25&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J25&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J25&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J25&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
         <x:v>4</x:v>
       </x:c>
@@ -3654,7 +3654,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac8ba386eaa9469a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1aa90f741855464a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3951,7 +3951,7 @@
         <x:v>Required U.S. H100-equivalents</x:v>
       </x:c>
       <x:c r="B12" s="18" t="n">
-        <x:f>B9*I11/B24</x:f>
+        <x:f>B9*I11/B25</x:f>
         <x:v>35979846.92445279</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
@@ -4167,32 +4167,45 @@
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="17" t="str">
-        <x:v>Compute-equivalent tokens / H100e / day</x:v>
-      </x:c>
-      <x:c r="B24" s="18" t="n">
-        <x:f>B16*B17*B18*B19*B23/(B20*B21*B22)</x:f>
+        <x:v>Personal-AI share of modeled inference</x:v>
+      </x:c>
+      <x:c r="B24" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C24" s="17" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D24" s="17" t="str">
+        <x:v>Scenario allocation to the target cohort; not an observed fleet share</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="17" t="str">
+        <x:v>Personal-AI compute-equivalent tokens / H100e / day</x:v>
+      </x:c>
+      <x:c r="B25" s="18" t="n">
+        <x:f>B16*B17*B18*B19*B23*B24/(B20*B21*B22)</x:f>
         <x:v>79793280</x:v>
       </x:c>
-      <x:c r="C24" s="17" t="str">
+      <x:c r="C25" s="17" t="str">
         <x:v>tokens/day</x:v>
       </x:c>
-      <x:c r="D24" s="17" t="str">
-        <x:v>Derived serving supply per H100-equivalent</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25"/>
+      <x:c r="D25" s="17" t="str">
+        <x:v>Derived serving supply available to the target cohort</x:v>
+      </x:c>
+    </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="9" t="str">
-        <x:v>QUARTERLY GROWTH MODEL</x:v>
+        <x:v>FORWARD CAPACITY PATH</x:v>
       </x:c>
       <x:c r="B26" s="9" t="str">
-        <x:v>QUARTERLY GROWTH MODEL</x:v>
+        <x:v>FORWARD CAPACITY PATH</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
-        <x:v>QUARTERLY GROWTH MODEL</x:v>
+        <x:v>FORWARD CAPACITY PATH</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
-        <x:v>QUARTERLY GROWTH MODEL</x:v>
+        <x:v>FORWARD CAPACITY PATH</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
@@ -4211,47 +4224,47 @@
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="17" t="str">
-        <x:v>Log-capacity acceleration</x:v>
+        <x:v>Pipeline log-capacity acceleration</x:v>
       </x:c>
       <x:c r="B28" s="27" t="n">
-        <x:f>SLOPE('Quarterly Model'!$G$7:$G$16,'Quarterly Model'!$A$7:$A$16)</x:f>
-        <x:v>-0.03112621365907439</x:v>
+        <x:f>SLOPE('Quarterly Model'!$G$17:$G$25,'Quarterly Model'!$A$17:$A$25)</x:f>
+        <x:v>0.003372652996279868</x:v>
       </x:c>
       <x:c r="C28" s="17" t="str">
         <x:v>log2 H100e / quarter²</x:v>
       </x:c>
       <x:c r="D28" s="17" t="str">
-        <x:v>Slope of observed quarterly log-growth rates</x:v>
+        <x:v>OLS slope of the published forward-path quarterly log-growth rates</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="17" t="str">
-        <x:v>Growth-rate intercept</x:v>
+        <x:v>Mean pipeline log growth</x:v>
       </x:c>
       <x:c r="B29" s="27" t="n">
-        <x:f>AVERAGE('Quarterly Model'!$G$7:$G$16)-B28*AVERAGE('Quarterly Model'!$A$7:$A$16)</x:f>
-        <x:v>0.7805896180694465</x:v>
+        <x:f>AVERAGE('Quarterly Model'!$G$17:$G$25)</x:f>
+        <x:v>0.24379055731655638</x:v>
       </x:c>
       <x:c r="C29" s="17" t="str">
         <x:v>log2 H100e / quarter</x:v>
       </x:c>
       <x:c r="D29" s="17" t="str">
-        <x:v>OLS intercept for observed quarterly growth</x:v>
+        <x:v>Mean quarterly log growth across the published forward path</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="17" t="str">
-        <x:v>Current smoothed velocity</x:v>
+        <x:v>First projected log growth</x:v>
       </x:c>
       <x:c r="B30" s="27" t="n">
-        <x:f>B29+B28*B10</x:f>
-        <x:v>0.4382012678196282</x:v>
+        <x:f>'Quarterly Model'!G17</x:f>
+        <x:v>0.3635456744374075</x:v>
       </x:c>
       <x:c r="C30" s="17" t="str">
         <x:v>log2 H100e / quarter</x:v>
       </x:c>
       <x:c r="D30" s="17" t="str">
-        <x:v>Intercept + acceleration × current quarter</x:v>
+        <x:v>Growth from the current snapshot to 2026-Q4</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
@@ -4260,7 +4273,7 @@
       </x:c>
       <x:c r="B31" s="17" t="n">
         <x:f>MATCH(1,'Quarterly Model'!$J$6:$J$25,0)</x:f>
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C31" s="17" t="str">
         <x:v>position</x:v>
@@ -4275,7 +4288,7 @@
       </x:c>
       <x:c r="B32" s="20" t="n">
         <x:f>INDEX('Quarterly Model'!$C$6:$C$25,B31-1)+(B12-INDEX('Quarterly Model'!$E$6:$E$25,B31-1))/(INDEX('Quarterly Model'!$E$6:$E$25,B31)-INDEX('Quarterly Model'!$E$6:$E$25,B31-1))*(INDEX('Quarterly Model'!$C$6:$C$25,B31)-INDEX('Quarterly Model'!$C$6:$C$25,B31-1))</x:f>
-        <x:v>46632.108708204854</x:v>
+        <x:v>46829.09207929863</x:v>
       </x:c>
       <x:c r="C32" s="17" t="str">
         <x:v>date</x:v>
@@ -4303,13 +4316,13 @@
         <x:v>Projected capability crossing</x:v>
       </x:c>
       <x:c r="B34" s="20" t="n">
-        <x:v>46668</x:v>
+        <x:v>46924</x:v>
       </x:c>
       <x:c r="C34" s="17" t="str">
         <x:v>date</x:v>
       </x:c>
       <x:c r="D34" s="17" t="str">
-        <x:v>Interpolated from the capability report card</x:v>
+        <x:v>First UTC day on which the capability report-card path reaches 60%</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
@@ -4318,7 +4331,7 @@
       </x:c>
       <x:c r="B35" s="20" t="n">
         <x:f>MAX(B32,B34)</x:f>
-        <x:v>46668</x:v>
+        <x:v>46924</x:v>
       </x:c>
       <x:c r="C35" s="17" t="str">
         <x:v>date</x:v>
@@ -4356,71 +4369,71 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
       <x:c r="D2" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
       <x:c r="E2" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
       <x:c r="F2" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>U.S. Operational AI-Compute Observations</x:v>
+        <x:v>U.S. AI-Compute Capacity Inputs</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>For each quarter cutoff, sum the latest H100-equivalent state for every Epoch-covered U.S. data center. 2026-Q3 is quarter-to-date through 2026-08-26.</x:v>
+        <x:v>Observed operational capacity through 2026-08-26; later rows use the expected/projected site states and dates in the same Epoch timeline snapshot.</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>For each quarter cutoff, sum the latest H100-equivalent state for every Epoch-covered U.S. data center. 2026-Q3 is quarter-to-date through 2026-08-26.</x:v>
+        <x:v>Observed operational capacity through 2026-08-26; later rows use the expected/projected site states and dates in the same Epoch timeline snapshot.</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>For each quarter cutoff, sum the latest H100-equivalent state for every Epoch-covered U.S. data center. 2026-Q3 is quarter-to-date through 2026-08-26.</x:v>
+        <x:v>Observed operational capacity through 2026-08-26; later rows use the expected/projected site states and dates in the same Epoch timeline snapshot.</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>For each quarter cutoff, sum the latest H100-equivalent state for every Epoch-covered U.S. data center. 2026-Q3 is quarter-to-date through 2026-08-26.</x:v>
+        <x:v>Observed operational capacity through 2026-08-26; later rows use the expected/projected site states and dates in the same Epoch timeline snapshot.</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>For each quarter cutoff, sum the latest H100-equivalent state for every Epoch-covered U.S. data center. 2026-Q3 is quarter-to-date through 2026-08-26.</x:v>
+        <x:v>Observed operational capacity through 2026-08-26; later rows use the expected/projected site states and dates in the same Epoch timeline snapshot.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>For each quarter cutoff, sum the latest H100-equivalent state for every Epoch-covered U.S. data center. 2026-Q3 is quarter-to-date through 2026-08-26.</x:v>
+        <x:v>Observed operational capacity through 2026-08-26; later rows use the expected/projected site states and dates in the same Epoch timeline snapshot.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>For each quarter cutoff, sum the latest H100-equivalent state for every Epoch-covered U.S. data center. 2026-Q3 is quarter-to-date through 2026-08-26.</x:v>
+        <x:v>Observed operational capacity through 2026-08-26; later rows use the expected/projected site states and dates in the same Epoch timeline snapshot.</x:v>
       </x:c>
     </x:row>
     <x:row r="4"/>
@@ -4438,7 +4451,7 @@
         <x:v>U.S. operational H100e</x:v>
       </x:c>
       <x:c r="E5" s="13" t="str">
-        <x:v>Operational sites</x:v>
+        <x:v>Included sites</x:v>
       </x:c>
       <x:c r="F5" s="13" t="str">
         <x:v>Evidence class</x:v>
@@ -4697,6 +4710,213 @@
         <x:v>Observed QTD</x:v>
       </x:c>
       <x:c r="G16" s="17" t="str">
+        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="23" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B17" s="23" t="str">
+        <x:v>2026-Q4</x:v>
+      </x:c>
+      <x:c r="C17" s="28" t="n">
+        <x:v>46387</x:v>
+      </x:c>
+      <x:c r="D17" s="29" t="n">
+        <x:v>17399770</x:v>
+      </x:c>
+      <x:c r="E17" s="29" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="F17" s="23" t="str">
+        <x:v>Epoch projected pipeline</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="str">
+        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="23" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B18" s="23" t="str">
+        <x:v>2027-Q1</x:v>
+      </x:c>
+      <x:c r="C18" s="28" t="n">
+        <x:v>46477</x:v>
+      </x:c>
+      <x:c r="D18" s="29" t="n">
+        <x:v>20368064</x:v>
+      </x:c>
+      <x:c r="E18" s="29" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="F18" s="23" t="str">
+        <x:v>Epoch projected pipeline</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="str">
+        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="23" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B19" s="23" t="str">
+        <x:v>2027-Q2</x:v>
+      </x:c>
+      <x:c r="C19" s="28" t="n">
+        <x:v>46568</x:v>
+      </x:c>
+      <x:c r="D19" s="29" t="n">
+        <x:v>21439292</x:v>
+      </x:c>
+      <x:c r="E19" s="29" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="F19" s="23" t="str">
+        <x:v>Epoch projected pipeline</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="str">
+        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="23" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B20" s="23" t="str">
+        <x:v>2027-Q3</x:v>
+      </x:c>
+      <x:c r="C20" s="28" t="n">
+        <x:v>46660</x:v>
+      </x:c>
+      <x:c r="D20" s="29" t="n">
+        <x:v>23242366</x:v>
+      </x:c>
+      <x:c r="E20" s="29" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="F20" s="23" t="str">
+        <x:v>Epoch projected pipeline</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="str">
+        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="23" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B21" s="23" t="str">
+        <x:v>2027-Q4</x:v>
+      </x:c>
+      <x:c r="C21" s="28" t="n">
+        <x:v>46752</x:v>
+      </x:c>
+      <x:c r="D21" s="29" t="n">
+        <x:v>30057691</x:v>
+      </x:c>
+      <x:c r="E21" s="29" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="F21" s="23" t="str">
+        <x:v>Epoch projected pipeline</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="str">
+        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="23" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B22" s="23" t="str">
+        <x:v>2028-Q1</x:v>
+      </x:c>
+      <x:c r="C22" s="28" t="n">
+        <x:v>46843</x:v>
+      </x:c>
+      <x:c r="D22" s="29" t="n">
+        <x:v>37048243</x:v>
+      </x:c>
+      <x:c r="E22" s="29" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="F22" s="23" t="str">
+        <x:v>Epoch projected pipeline</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="str">
+        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="23" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B23" s="23" t="str">
+        <x:v>2028-Q2</x:v>
+      </x:c>
+      <x:c r="C23" s="28" t="n">
+        <x:v>46934</x:v>
+      </x:c>
+      <x:c r="D23" s="29" t="n">
+        <x:v>46037632</x:v>
+      </x:c>
+      <x:c r="E23" s="29" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="F23" s="23" t="str">
+        <x:v>Epoch projected pipeline</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="str">
+        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="23" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B24" s="23" t="str">
+        <x:v>2028-Q3</x:v>
+      </x:c>
+      <x:c r="C24" s="28" t="n">
+        <x:v>47026</x:v>
+      </x:c>
+      <x:c r="D24" s="29" t="n">
+        <x:v>47106859</x:v>
+      </x:c>
+      <x:c r="E24" s="29" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="F24" s="23" t="str">
+        <x:v>Epoch projected pipeline</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="str">
+        <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="23" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B25" s="23" t="str">
+        <x:v>2028-Q4</x:v>
+      </x:c>
+      <x:c r="C25" s="28" t="n">
+        <x:v>47118</x:v>
+      </x:c>
+      <x:c r="D25" s="29" t="n">
+        <x:v>61887051</x:v>
+      </x:c>
+      <x:c r="E25" s="29" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="F25" s="23" t="str">
+        <x:v>Epoch projected pipeline</x:v>
+      </x:c>
+      <x:c r="G25" s="23" t="str">
         <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
       </x:c>
     </x:row>
@@ -4707,7 +4927,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09fdb693ea1e44ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5990f97ea774270"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4825,7 +5045,7 @@
         <x:v>Dataset scope, H100e convention, coverage, and uncertainty</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+    <x:row r="7" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A7" s="17" t="str">
         <x:v>SRC-002</x:v>
       </x:c>
@@ -4842,7 +5062,7 @@
         <x:v>https://epoch.ai/data/data_centers/data_center_timelines.csv</x:v>
       </x:c>
       <x:c r="F7" s="17" t="str">
-        <x:v>Quarterly U.S. operational H100e reconstructed from latest site state at each cutoff</x:v>
+        <x:v>Observed quarters use latest operational state at each cutoff; forward quarters use the latest expected/projected state dated by each cutoff</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -4922,7 +5142,7 @@
         <x:v>https://diffuse-personal-ai-countdown.buddywilliams.chatgpt.site/?report=capability</x:v>
       </x:c>
       <x:c r="F11" s="17" t="str">
-        <x:v>Capability crosses 60% by interpolation around 2027-10-08</x:v>
+        <x:v>Capability first reaches 60% on the daily site path on 2028-06-20</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4932,7 +5152,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c71e88d68d84bc2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd156bc7772fb4a2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Set personal AI inference share to 50 percent
</commit_message>
<xml_diff>
--- a/data/reports/personal-ai-compute-report-card.xlsx
+++ b/data/reports/personal-ai-compute-report-card.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2655e89dff2343af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compute Report Card" sheetId="2" r:id="R77f515a337244c5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="3" r:id="R25796c800c7c470e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R80aaaa569da04f06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" r:id="R125e40b3a190432c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rc68bc68b5a1c4fb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4ad33934139b4500"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compute Report Card" sheetId="2" r:id="Re98b9d51da3d4e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="3" r:id="R48a1feb01b7345b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Ra4938a3d59374b6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" r:id="R368602b363824e18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R0a5e5e32eebd45b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -298,7 +298,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>Published U.S. buildout pipeline reaches the threshold in 2028</a:t>
+              <a:t>Published U.S. buildout pipeline approaches the threshold through 2028</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -470,7 +470,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8a28e480823e4a78"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc5bdbe21adb0459a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -920,7 +920,7 @@
     <x:row r="6">
       <x:c r="A6" s="55" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
-        <x:v>0.37587725229616675</x:v>
+        <x:v>0.18793862614808338</x:v>
       </x:c>
       <x:c r="D6" s="56" t="n">
         <x:f>'Quarterly Model'!E16</x:f>
@@ -930,11 +930,11 @@
       <x:c r="F6" s="57"/>
       <x:c r="G6" s="56" t="n">
         <x:f>'Quarterly Model'!I16</x:f>
-        <x:v>64425361.043562986</x:v>
+        <x:v>32212680.521781493</x:v>
       </x:c>
       <x:c r="J6" s="58" t="n">
         <x:f>'Assumptions'!B32</x:f>
-        <x:v>46829.09207929863</x:v>
+        <x:v>47168.12398813577</x:v>
       </x:c>
       <x:c r="M6" s="54" t="str">
         <x:f>'Quarterly Model'!L16</x:f>
@@ -1014,11 +1014,11 @@
       </x:c>
       <x:c r="C14" s="31" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
-        <x:v>0.37587725229616675</x:v>
+        <x:v>0.18793862614808338</x:v>
       </x:c>
       <x:c r="D14" s="20" t="n">
         <x:f>'Assumptions'!B32</x:f>
-        <x:v>46829.09207929863</x:v>
+        <x:v>47168.12398813577</x:v>
       </x:c>
       <x:c r="E14" s="17" t="str">
         <x:v>Waiting</x:v>
@@ -1037,7 +1037,7 @@
       <x:c r="C15" s="24"/>
       <x:c r="D15" s="59" t="n">
         <x:f>'Assumptions'!B35</x:f>
-        <x:v>46924</x:v>
+        <x:v>47168.12398813577</x:v>
       </x:c>
       <x:c r="E15" s="24" t="str">
         <x:v>Later crossing</x:v>
@@ -1077,7 +1077,7 @@
       </x:c>
       <x:c r="B20" s="19" t="n">
         <x:f>'Quarterly Model'!J6</x:f>
-        <x:v>0.00682782226716592</x:v>
+        <x:v>0.00341391113358296</x:v>
       </x:c>
       <x:c r="C20" s="19" t="n">
         <x:f>1</x:f>
@@ -1091,7 +1091,7 @@
       </x:c>
       <x:c r="B21" s="19" t="n">
         <x:f>'Quarterly Model'!J7</x:f>
-        <x:v>0.01320844974682248</x:v>
+        <x:v>0.00660422487341124</x:v>
       </x:c>
       <x:c r="C21" s="19" t="n">
         <x:f>1</x:f>
@@ -1105,7 +1105,7 @@
       </x:c>
       <x:c r="B22" s="19" t="n">
         <x:f>'Quarterly Model'!J8</x:f>
-        <x:v>0.020071791898291506</x:v>
+        <x:v>0.010035895949145753</x:v>
       </x:c>
       <x:c r="C22" s="19" t="n">
         <x:f>1</x:f>
@@ -1119,7 +1119,7 @@
       </x:c>
       <x:c r="B23" s="19" t="n">
         <x:f>'Quarterly Model'!J9</x:f>
-        <x:v>0.02814028092242638</x:v>
+        <x:v>0.01407014046121319</x:v>
       </x:c>
       <x:c r="C23" s="19" t="n">
         <x:f>1</x:f>
@@ -1133,7 +1133,7 @@
       </x:c>
       <x:c r="B24" s="19" t="n">
         <x:f>'Quarterly Model'!J10</x:f>
-        <x:v>0.037555468283042195</x:v>
+        <x:v>0.018777734141521098</x:v>
       </x:c>
       <x:c r="C24" s="19" t="n">
         <x:f>1</x:f>
@@ -1147,7 +1147,7 @@
       </x:c>
       <x:c r="B25" s="19" t="n">
         <x:f>'Quarterly Model'!J11</x:f>
-        <x:v>0.06633924833009283</x:v>
+        <x:v>0.033169624165046416</x:v>
       </x:c>
       <x:c r="C25" s="19" t="n">
         <x:f>1</x:f>
@@ -1161,7 +1161,7 @@
       </x:c>
       <x:c r="B26" s="19" t="n">
         <x:f>'Quarterly Model'!J12</x:f>
-        <x:v>0.08726162750476324</x:v>
+        <x:v>0.04363081375238162</x:v>
       </x:c>
       <x:c r="C26" s="19" t="n">
         <x:f>1</x:f>
@@ -1175,7 +1175,7 @@
       </x:c>
       <x:c r="B27" s="19" t="n">
         <x:f>'Quarterly Model'!J13</x:f>
-        <x:v>0.14706496698305438</x:v>
+        <x:v>0.07353248349152719</x:v>
       </x:c>
       <x:c r="C27" s="19" t="n">
         <x:f>1</x:f>
@@ -1189,7 +1189,7 @@
       </x:c>
       <x:c r="B28" s="19" t="n">
         <x:f>'Quarterly Model'!J14</x:f>
-        <x:v>0.17513398579018094</x:v>
+        <x:v>0.08756699289509047</x:v>
       </x:c>
       <x:c r="C28" s="19" t="n">
         <x:f>1</x:f>
@@ -1203,7 +1203,7 @@
       </x:c>
       <x:c r="B29" s="19" t="n">
         <x:f>'Quarterly Model'!J15</x:f>
-        <x:v>0.31194838109141576</x:v>
+        <x:v>0.15597419054570788</x:v>
       </x:c>
       <x:c r="C29" s="19" t="n">
         <x:f>1</x:f>
@@ -1217,7 +1217,7 @@
       </x:c>
       <x:c r="B30" s="19" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
-        <x:v>0.37587725229616675</x:v>
+        <x:v>0.18793862614808338</x:v>
       </x:c>
       <x:c r="C30" s="19" t="n">
         <x:f>1</x:f>
@@ -1231,7 +1231,7 @@
       </x:c>
       <x:c r="B31" s="19" t="n">
         <x:f>'Quarterly Model'!J17</x:f>
-        <x:v>0.48359766611943783</x:v>
+        <x:v>0.24179883305971892</x:v>
       </x:c>
       <x:c r="C31" s="19" t="n">
         <x:f>1</x:f>
@@ -1245,7 +1245,7 @@
       </x:c>
       <x:c r="B32" s="19" t="n">
         <x:f>'Quarterly Model'!J18</x:f>
-        <x:v>0.5660964606872011</x:v>
+        <x:v>0.28304823034360055</x:v>
       </x:c>
       <x:c r="C32" s="19" t="n">
         <x:f>1</x:f>
@@ -1259,7 +1259,7 @@
       </x:c>
       <x:c r="B33" s="19" t="n">
         <x:f>'Quarterly Model'!J19</x:f>
-        <x:v>0.5958694611740921</x:v>
+        <x:v>0.29793473058704606</x:v>
       </x:c>
       <x:c r="C33" s="19" t="n">
         <x:f>1</x:f>
@@ -1273,7 +1273,7 @@
       </x:c>
       <x:c r="B34" s="19" t="n">
         <x:f>'Quarterly Model'!J20</x:f>
-        <x:v>0.6459829039518208</x:v>
+        <x:v>0.3229914519759104</x:v>
       </x:c>
       <x:c r="C34" s="19" t="n">
         <x:f>1</x:f>
@@ -1287,7 +1287,7 @@
       </x:c>
       <x:c r="B35" s="19" t="n">
         <x:f>'Quarterly Model'!J21</x:f>
-        <x:v>0.8354035263994427</x:v>
+        <x:v>0.41770176319972135</x:v>
       </x:c>
       <x:c r="C35" s="19" t="n">
         <x:f>1</x:f>
@@ -1301,7 +1301,7 @@
       </x:c>
       <x:c r="B36" s="19" t="n">
         <x:f>'Quarterly Model'!J22</x:f>
-        <x:v>1</x:v>
+        <x:v>0.5148471459285324</x:v>
       </x:c>
       <x:c r="C36" s="19" t="n">
         <x:f>1</x:f>
@@ -1315,7 +1315,7 @@
       </x:c>
       <x:c r="B37" s="19" t="n">
         <x:f>'Quarterly Model'!J23</x:f>
-        <x:v>1</x:v>
+        <x:v>0.6397697035324474</x:v>
       </x:c>
       <x:c r="C37" s="19" t="n">
         <x:f>1</x:f>
@@ -1329,7 +1329,7 @@
       </x:c>
       <x:c r="B38" s="19" t="n">
         <x:f>'Quarterly Model'!J24</x:f>
-        <x:v>1</x:v>
+        <x:v>0.6546283965425242</x:v>
       </x:c>
       <x:c r="C38" s="19" t="n">
         <x:f>1</x:f>
@@ -1343,7 +1343,7 @@
       </x:c>
       <x:c r="B39" s="19" t="n">
         <x:f>'Quarterly Model'!J25</x:f>
-        <x:v>1</x:v>
+        <x:v>0.860023822918769</x:v>
       </x:c>
       <x:c r="C39" s="19" t="n">
         <x:f>1</x:f>
@@ -1356,7 +1356,7 @@
         <x:v>Interpretation</x:v>
       </x:c>
       <x:c r="B41" s="17" t="str">
-        <x:v>Current U.S. operational capacity supports about 64 million high-autonomy users under the base serving envelope—37.6% of the 171.4 million-user threshold.</x:v>
+        <x:v>At the 50% personal-AI inference allocation, current U.S. operational capacity supports about 32 million high-autonomy users—18.8% of the 171.4 million-user threshold.</x:v>
       </x:c>
       <x:c r="C41" s="17"/>
       <x:c r="D41" s="17"/>
@@ -1416,7 +1416,7 @@
         <x:v>Caution</x:v>
       </x:c>
       <x:c r="B44" s="17" t="str">
-        <x:v>Epoch covers publicly tracked large sites rather than the full U.S. fleet. Project timing and quantity are uncertain. The editable base case allocates 100% of modeled inference supply to this personal-AI cohort.</x:v>
+        <x:v>Epoch covers publicly tracked large sites rather than the full U.S. fleet. Project timing and quantity are uncertain. The editable base case allocates 50% of modeled inference supply to this personal-AI cohort.</x:v>
       </x:c>
       <x:c r="C44" s="17"/>
       <x:c r="D44" s="17"/>
@@ -1453,7 +1453,7 @@
     <x:mergeCell ref="B44:N44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf63d864810a34034"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2acf7977cf74b65"/>
 </x:worksheet>
 </file>
 
@@ -2246,166 +2246,166 @@
       </x:c>
       <x:c r="C6" s="46" t="n">
         <x:f>'Quarterly Model'!J6</x:f>
-        <x:v>0.00682782226716592</x:v>
+        <x:v>0.00341391113358296</x:v>
       </x:c>
       <x:c r="D6" s="46" t="str">
         <x:f>'Quarterly Model'!K6</x:f>
       </x:c>
       <x:c r="E6" s="46" t="n">
         <x:f>'Quarterly Model'!J7</x:f>
-        <x:v>0.01320844974682248</x:v>
+        <x:v>0.00660422487341124</x:v>
       </x:c>
       <x:c r="F6" s="46" t="n">
         <x:f>'Quarterly Model'!K7</x:f>
-        <x:v>0.006380627479656559</x:v>
+        <x:v>0.0031903137398282795</x:v>
       </x:c>
       <x:c r="G6" s="46" t="n">
         <x:f>'Quarterly Model'!J8</x:f>
-        <x:v>0.020071791898291506</x:v>
+        <x:v>0.010035895949145753</x:v>
       </x:c>
       <x:c r="H6" s="46" t="n">
         <x:f>'Quarterly Model'!K8</x:f>
-        <x:v>0.006863342151469026</x:v>
+        <x:v>0.003431671075734513</x:v>
       </x:c>
       <x:c r="I6" s="46" t="n">
         <x:f>'Quarterly Model'!J9</x:f>
-        <x:v>0.02814028092242638</x:v>
+        <x:v>0.01407014046121319</x:v>
       </x:c>
       <x:c r="J6" s="46" t="n">
         <x:f>'Quarterly Model'!K9</x:f>
-        <x:v>0.008068489024134873</x:v>
+        <x:v>0.004034244512067436</x:v>
       </x:c>
       <x:c r="K6" s="46" t="n">
         <x:f>'Quarterly Model'!J10</x:f>
-        <x:v>0.037555468283042195</x:v>
+        <x:v>0.018777734141521098</x:v>
       </x:c>
       <x:c r="L6" s="46" t="n">
         <x:f>'Quarterly Model'!K10</x:f>
-        <x:v>0.009415187360615817</x:v>
+        <x:v>0.0047075936803079085</x:v>
       </x:c>
       <x:c r="M6" s="46" t="n">
         <x:f>'Quarterly Model'!J11</x:f>
-        <x:v>0.06633924833009283</x:v>
+        <x:v>0.033169624165046416</x:v>
       </x:c>
       <x:c r="N6" s="46" t="n">
         <x:f>'Quarterly Model'!K11</x:f>
-        <x:v>0.028783780047050636</x:v>
+        <x:v>0.014391890023525318</x:v>
       </x:c>
       <x:c r="O6" s="46" t="n">
         <x:f>'Quarterly Model'!J12</x:f>
-        <x:v>0.08726162750476324</x:v>
+        <x:v>0.04363081375238162</x:v>
       </x:c>
       <x:c r="P6" s="46" t="n">
         <x:f>'Quarterly Model'!K12</x:f>
-        <x:v>0.020922379174670408</x:v>
+        <x:v>0.010461189587335204</x:v>
       </x:c>
       <x:c r="Q6" s="46" t="n">
         <x:f>'Quarterly Model'!J13</x:f>
-        <x:v>0.14706496698305438</x:v>
+        <x:v>0.07353248349152719</x:v>
       </x:c>
       <x:c r="R6" s="46" t="n">
         <x:f>'Quarterly Model'!K13</x:f>
-        <x:v>0.05980333947829114</x:v>
+        <x:v>0.02990166973914557</x:v>
       </x:c>
       <x:c r="S6" s="46" t="n">
         <x:f>'Quarterly Model'!J14</x:f>
-        <x:v>0.17513398579018094</x:v>
+        <x:v>0.08756699289509047</x:v>
       </x:c>
       <x:c r="T6" s="46" t="n">
         <x:f>'Quarterly Model'!K14</x:f>
-        <x:v>0.02806901880712656</x:v>
+        <x:v>0.01403450940356328</x:v>
       </x:c>
       <x:c r="U6" s="46" t="n">
         <x:f>'Quarterly Model'!J15</x:f>
-        <x:v>0.31194838109141576</x:v>
+        <x:v>0.15597419054570788</x:v>
       </x:c>
       <x:c r="V6" s="46" t="n">
         <x:f>'Quarterly Model'!K15</x:f>
-        <x:v>0.13681439530123482</x:v>
+        <x:v>0.06840719765061741</x:v>
       </x:c>
       <x:c r="W6" s="46" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
-        <x:v>0.37587725229616675</x:v>
+        <x:v>0.18793862614808338</x:v>
       </x:c>
       <x:c r="X6" s="46" t="n">
         <x:f>'Quarterly Model'!K16</x:f>
-        <x:v>0.06392887120475099</x:v>
+        <x:v>0.031964435602375496</x:v>
       </x:c>
       <x:c r="Y6" s="34" t="n">
         <x:f>'Quarterly Model'!J17</x:f>
-        <x:v>0.48359766611943783</x:v>
+        <x:v>0.24179883305971892</x:v>
       </x:c>
       <x:c r="Z6" s="34" t="n">
         <x:f>'Quarterly Model'!K17</x:f>
-        <x:v>0.10772041382327108</x:v>
+        <x:v>0.05386020691163554</x:v>
       </x:c>
       <x:c r="AA6" s="34" t="n">
         <x:f>'Quarterly Model'!J18</x:f>
-        <x:v>0.5660964606872011</x:v>
+        <x:v>0.28304823034360055</x:v>
       </x:c>
       <x:c r="AB6" s="34" t="n">
         <x:f>'Quarterly Model'!K18</x:f>
-        <x:v>0.08249879456776327</x:v>
+        <x:v>0.041249397283881634</x:v>
       </x:c>
       <x:c r="AC6" s="34" t="n">
         <x:f>'Quarterly Model'!J19</x:f>
-        <x:v>0.5958694611740921</x:v>
+        <x:v>0.29793473058704606</x:v>
       </x:c>
       <x:c r="AD6" s="34" t="n">
         <x:f>'Quarterly Model'!K19</x:f>
-        <x:v>0.02977300048689102</x:v>
+        <x:v>0.01488650024344551</x:v>
       </x:c>
       <x:c r="AE6" s="34" t="n">
         <x:f>'Quarterly Model'!J20</x:f>
-        <x:v>0.6459829039518208</x:v>
+        <x:v>0.3229914519759104</x:v>
       </x:c>
       <x:c r="AF6" s="34" t="n">
         <x:f>'Quarterly Model'!K20</x:f>
-        <x:v>0.05011344277772867</x:v>
+        <x:v>0.025056721388864334</x:v>
       </x:c>
       <x:c r="AG6" s="34" t="n">
         <x:f>'Quarterly Model'!J21</x:f>
-        <x:v>0.8354035263994427</x:v>
+        <x:v>0.41770176319972135</x:v>
       </x:c>
       <x:c r="AH6" s="34" t="n">
         <x:f>'Quarterly Model'!K21</x:f>
-        <x:v>0.18942062244762192</x:v>
+        <x:v>0.09471031122381096</x:v>
       </x:c>
       <x:c r="AI6" s="34" t="n">
         <x:f>'Quarterly Model'!J22</x:f>
-        <x:v>1</x:v>
+        <x:v>0.5148471459285324</x:v>
       </x:c>
       <x:c r="AJ6" s="34" t="n">
         <x:f>'Quarterly Model'!K22</x:f>
-        <x:v>0.1645964736005573</x:v>
+        <x:v>0.09714538272881107</x:v>
       </x:c>
       <x:c r="AK6" s="34" t="n">
         <x:f>'Quarterly Model'!J23</x:f>
-        <x:v>1</x:v>
+        <x:v>0.6397697035324474</x:v>
       </x:c>
       <x:c r="AL6" s="34" t="n">
         <x:f>'Quarterly Model'!K23</x:f>
-        <x:v>0</x:v>
+        <x:v>0.12492255760391502</x:v>
       </x:c>
       <x:c r="AM6" s="34" t="n">
         <x:f>'Quarterly Model'!J24</x:f>
-        <x:v>1</x:v>
+        <x:v>0.6546283965425242</x:v>
       </x:c>
       <x:c r="AN6" s="34" t="n">
         <x:f>'Quarterly Model'!K24</x:f>
-        <x:v>0</x:v>
+        <x:v>0.014858693010076807</x:v>
       </x:c>
       <x:c r="AO6" s="34" t="n">
         <x:f>'Quarterly Model'!J25</x:f>
-        <x:v>1</x:v>
+        <x:v>0.860023822918769</x:v>
       </x:c>
       <x:c r="AP6" s="34" t="n">
         <x:f>'Quarterly Model'!K25</x:f>
-        <x:v>0</x:v>
+        <x:v>0.20539542637624475</x:v>
       </x:c>
       <x:c r="AQ6" s="31" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
-        <x:v>0.37587725229616675</x:v>
+        <x:v>0.18793862614808338</x:v>
       </x:c>
       <x:c r="AR6" s="31" t="str">
         <x:f>'Quarterly Model'!L16</x:f>
@@ -2417,7 +2417,7 @@
       </x:c>
       <x:c r="AT6" s="20" t="n">
         <x:f>'Assumptions'!B32</x:f>
-        <x:v>46829.09207929863</x:v>
+        <x:v>47168.12398813577</x:v>
       </x:c>
       <x:c r="AU6" s="27" t="n">
         <x:f>'Assumptions'!B30</x:f>
@@ -2675,15 +2675,15 @@
       </x:c>
       <x:c r="H6" s="30" t="n">
         <x:f>E6*'Assumptions'!$B$25</x:f>
-        <x:v>19602336337920</x:v>
+        <x:v>9801168168960</x:v>
       </x:c>
       <x:c r="I6" s="18" t="n">
         <x:f>H6/'Assumptions'!$I$11</x:f>
-        <x:v>1170288.7365922388</x:v>
+        <x:v>585144.3682961194</x:v>
       </x:c>
       <x:c r="J6" s="31" t="n">
         <x:f>MIN(1,I6/'Assumptions'!$B$9)</x:f>
-        <x:v>0.00682782226716592</x:v>
+        <x:v>0.00341391113358296</x:v>
       </x:c>
       <x:c r="K6" s="31" t="str">
         <x:f>""</x:f>
@@ -2724,19 +2724,19 @@
       </x:c>
       <x:c r="H7" s="30" t="n">
         <x:f>E7*'Assumptions'!$B$25</x:f>
-        <x:v>37920798800640</x:v>
+        <x:v>18960399400320</x:v>
       </x:c>
       <x:c r="I7" s="18" t="n">
         <x:f>H7/'Assumptions'!$I$11</x:f>
-        <x:v>2263928.286605373</x:v>
+        <x:v>1131964.1433026865</x:v>
       </x:c>
       <x:c r="J7" s="31" t="n">
         <x:f>MIN(1,I7/'Assumptions'!$B$9)</x:f>
-        <x:v>0.01320844974682248</x:v>
+        <x:v>0.00660422487341124</x:v>
       </x:c>
       <x:c r="K7" s="31" t="n">
         <x:f>J7-J6</x:f>
-        <x:v>0.006380627479656559</x:v>
+        <x:v>0.0031903137398282795</x:v>
       </x:c>
       <x:c r="L7" s="17" t="str">
         <x:f>IF(J7&gt;='Assumptions'!$G$16,"A",IF(J7&gt;='Assumptions'!$G$17,"B",IF(J7&gt;='Assumptions'!$G$18,"C",IF(J7&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -2774,19 +2774,19 @@
       </x:c>
       <x:c r="H8" s="30" t="n">
         <x:f>E8*'Assumptions'!$B$25</x:f>
-        <x:v>57625110950400</x:v>
+        <x:v>28812555475200</x:v>
       </x:c>
       <x:c r="I8" s="18" t="n">
         <x:f>H8/'Assumptions'!$I$11</x:f>
-        <x:v>3440305.131367164</x:v>
+        <x:v>1720152.565683582</x:v>
       </x:c>
       <x:c r="J8" s="31" t="n">
         <x:f>MIN(1,I8/'Assumptions'!$B$9)</x:f>
-        <x:v>0.020071791898291506</x:v>
+        <x:v>0.010035895949145753</x:v>
       </x:c>
       <x:c r="K8" s="31" t="n">
         <x:f>J8-J7</x:f>
-        <x:v>0.006863342151469026</x:v>
+        <x:v>0.003431671075734513</x:v>
       </x:c>
       <x:c r="L8" s="17" t="str">
         <x:f>IF(J8&gt;='Assumptions'!$G$16,"A",IF(J8&gt;='Assumptions'!$G$17,"B",IF(J8&gt;='Assumptions'!$G$18,"C",IF(J8&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -2824,19 +2824,19 @@
       </x:c>
       <x:c r="H9" s="30" t="n">
         <x:f>E9*'Assumptions'!$B$25</x:f>
-        <x:v>80789339514240</x:v>
+        <x:v>40394669757120</x:v>
       </x:c>
       <x:c r="I9" s="18" t="n">
         <x:f>H9/'Assumptions'!$I$11</x:f>
-        <x:v>4823244.150103881</x:v>
+        <x:v>2411622.0750519405</x:v>
       </x:c>
       <x:c r="J9" s="31" t="n">
         <x:f>MIN(1,I9/'Assumptions'!$B$9)</x:f>
-        <x:v>0.02814028092242638</x:v>
+        <x:v>0.01407014046121319</x:v>
       </x:c>
       <x:c r="K9" s="31" t="n">
         <x:f>J9-J8</x:f>
-        <x:v>0.008068489024134873</x:v>
+        <x:v>0.004034244512067436</x:v>
       </x:c>
       <x:c r="L9" s="17" t="str">
         <x:f>IF(J9&gt;='Assumptions'!$G$16,"A",IF(J9&gt;='Assumptions'!$G$17,"B",IF(J9&gt;='Assumptions'!$G$18,"C",IF(J9&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -2874,19 +2874,19 @@
       </x:c>
       <x:c r="H10" s="30" t="n">
         <x:f>E10*'Assumptions'!$B$25</x:f>
-        <x:v>107819871667200</x:v>
+        <x:v>53909935833600</x:v>
       </x:c>
       <x:c r="I10" s="18" t="n">
         <x:f>H10/'Assumptions'!$I$11</x:f>
-        <x:v>6437007.2637134325</x:v>
+        <x:v>3218503.6318567162</x:v>
       </x:c>
       <x:c r="J10" s="31" t="n">
         <x:f>MIN(1,I10/'Assumptions'!$B$9)</x:f>
-        <x:v>0.037555468283042195</x:v>
+        <x:v>0.018777734141521098</x:v>
       </x:c>
       <x:c r="K10" s="31" t="n">
         <x:f>J10-J9</x:f>
-        <x:v>0.009415187360615817</x:v>
+        <x:v>0.0047075936803079085</x:v>
       </x:c>
       <x:c r="L10" s="17" t="str">
         <x:f>IF(J10&gt;='Assumptions'!$G$16,"A",IF(J10&gt;='Assumptions'!$G$17,"B",IF(J10&gt;='Assumptions'!$G$18,"C",IF(J10&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -2924,19 +2924,19 @@
       </x:c>
       <x:c r="H11" s="30" t="n">
         <x:f>E11*'Assumptions'!$B$25</x:f>
-        <x:v>190456664993280</x:v>
+        <x:v>95228332496640</x:v>
       </x:c>
       <x:c r="I11" s="18" t="n">
         <x:f>H11/'Assumptions'!$I$11</x:f>
-        <x:v>11370547.16377791</x:v>
+        <x:v>5685273.581888955</x:v>
       </x:c>
       <x:c r="J11" s="31" t="n">
         <x:f>MIN(1,I11/'Assumptions'!$B$9)</x:f>
-        <x:v>0.06633924833009283</x:v>
+        <x:v>0.033169624165046416</x:v>
       </x:c>
       <x:c r="K11" s="31" t="n">
         <x:f>J11-J10</x:f>
-        <x:v>0.028783780047050636</x:v>
+        <x:v>0.014391890023525318</x:v>
       </x:c>
       <x:c r="L11" s="17" t="str">
         <x:f>IF(J11&gt;='Assumptions'!$G$16,"A",IF(J11&gt;='Assumptions'!$G$17,"B",IF(J11&gt;='Assumptions'!$G$18,"C",IF(J11&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -2974,19 +2974,19 @@
       </x:c>
       <x:c r="H12" s="30" t="n">
         <x:f>E12*'Assumptions'!$B$25</x:f>
-        <x:v>250523769484800</x:v>
+        <x:v>125261884742400</x:v>
       </x:c>
       <x:c r="I12" s="18" t="n">
         <x:f>H12/'Assumptions'!$I$11</x:f>
-        <x:v>14956642.954316419</x:v>
+        <x:v>7478321.477158209</x:v>
       </x:c>
       <x:c r="J12" s="31" t="n">
         <x:f>MIN(1,I12/'Assumptions'!$B$9)</x:f>
-        <x:v>0.08726162750476324</x:v>
+        <x:v>0.04363081375238162</x:v>
       </x:c>
       <x:c r="K12" s="31" t="n">
         <x:f>J12-J11</x:f>
-        <x:v>0.020922379174670408</x:v>
+        <x:v>0.010461189587335204</x:v>
       </x:c>
       <x:c r="L12" s="17" t="str">
         <x:f>IF(J12&gt;='Assumptions'!$G$16,"A",IF(J12&gt;='Assumptions'!$G$17,"B",IF(J12&gt;='Assumptions'!$G$18,"C",IF(J12&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3024,19 +3024,19 @@
       </x:c>
       <x:c r="H13" s="30" t="n">
         <x:f>E13*'Assumptions'!$B$25</x:f>
-        <x:v>422216166960000</x:v>
+        <x:v>211108083480000</x:v>
       </x:c>
       <x:c r="I13" s="18" t="n">
         <x:f>H13/'Assumptions'!$I$11</x:f>
-        <x:v>25206935.340895522</x:v>
+        <x:v>12603467.670447761</x:v>
       </x:c>
       <x:c r="J13" s="31" t="n">
         <x:f>MIN(1,I13/'Assumptions'!$B$9)</x:f>
-        <x:v>0.14706496698305438</x:v>
+        <x:v>0.07353248349152719</x:v>
       </x:c>
       <x:c r="K13" s="31" t="n">
         <x:f>J13-J12</x:f>
-        <x:v>0.05980333947829114</x:v>
+        <x:v>0.02990166973914557</x:v>
       </x:c>
       <x:c r="L13" s="17" t="str">
         <x:f>IF(J13&gt;='Assumptions'!$G$16,"A",IF(J13&gt;='Assumptions'!$G$17,"B",IF(J13&gt;='Assumptions'!$G$18,"C",IF(J13&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3074,19 +3074,19 @@
       </x:c>
       <x:c r="H14" s="30" t="n">
         <x:f>E14*'Assumptions'!$B$25</x:f>
-        <x:v>502800916504320</x:v>
+        <x:v>251400458252160</x:v>
       </x:c>
       <x:c r="I14" s="18" t="n">
         <x:f>H14/'Assumptions'!$I$11</x:f>
-        <x:v>30017965.164437015</x:v>
+        <x:v>15008982.582218507</x:v>
       </x:c>
       <x:c r="J14" s="31" t="n">
         <x:f>MIN(1,I14/'Assumptions'!$B$9)</x:f>
-        <x:v>0.17513398579018094</x:v>
+        <x:v>0.08756699289509047</x:v>
       </x:c>
       <x:c r="K14" s="31" t="n">
         <x:f>J14-J13</x:f>
-        <x:v>0.02806901880712656</x:v>
+        <x:v>0.01403450940356328</x:v>
       </x:c>
       <x:c r="L14" s="17" t="str">
         <x:f>IF(J14&gt;='Assumptions'!$G$16,"A",IF(J14&gt;='Assumptions'!$G$17,"B",IF(J14&gt;='Assumptions'!$G$18,"C",IF(J14&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3124,19 +3124,19 @@
       </x:c>
       <x:c r="H15" s="30" t="n">
         <x:f>E15*'Assumptions'!$B$25</x:f>
-        <x:v>895588204694400</x:v>
+        <x:v>447794102347200</x:v>
       </x:c>
       <x:c r="I15" s="18" t="n">
         <x:f>H15/'Assumptions'!$I$11</x:f>
-        <x:v>53467952.51906866</x:v>
+        <x:v>26733976.25953433</x:v>
       </x:c>
       <x:c r="J15" s="31" t="n">
         <x:f>MIN(1,I15/'Assumptions'!$B$9)</x:f>
-        <x:v>0.31194838109141576</x:v>
+        <x:v>0.15597419054570788</x:v>
       </x:c>
       <x:c r="K15" s="31" t="n">
         <x:f>J15-J14</x:f>
-        <x:v>0.13681439530123482</x:v>
+        <x:v>0.06840719765061741</x:v>
       </x:c>
       <x:c r="L15" s="17" t="str">
         <x:f>IF(J15&gt;='Assumptions'!$G$16,"A",IF(J15&gt;='Assumptions'!$G$17,"B",IF(J15&gt;='Assumptions'!$G$18,"C",IF(J15&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3174,19 +3174,19 @@
       </x:c>
       <x:c r="H16" s="30" t="n">
         <x:f>E16*'Assumptions'!$B$25</x:f>
-        <x:v>1079124797479680</x:v>
+        <x:v>539562398739840</x:v>
       </x:c>
       <x:c r="I16" s="18" t="n">
         <x:f>H16/'Assumptions'!$I$11</x:f>
-        <x:v>64425361.043562986</x:v>
+        <x:v>32212680.521781493</x:v>
       </x:c>
       <x:c r="J16" s="31" t="n">
         <x:f>MIN(1,I16/'Assumptions'!$B$9)</x:f>
-        <x:v>0.37587725229616675</x:v>
+        <x:v>0.18793862614808338</x:v>
       </x:c>
       <x:c r="K16" s="31" t="n">
         <x:f>J16-J15</x:f>
-        <x:v>0.06392887120475099</x:v>
+        <x:v>0.031964435602375496</x:v>
       </x:c>
       <x:c r="L16" s="17" t="str">
         <x:f>IF(J16&gt;='Assumptions'!$G$16,"A",IF(J16&gt;='Assumptions'!$G$17,"B",IF(J16&gt;='Assumptions'!$G$18,"C",IF(J16&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3224,19 +3224,19 @@
       </x:c>
       <x:c r="H17" s="33" t="n">
         <x:f>E17*'Assumptions'!$B$25</x:f>
-        <x:v>1388384719545600</x:v>
+        <x:v>694192359772800</x:v>
       </x:c>
       <x:c r="I17" s="29" t="n">
         <x:f>H17/'Assumptions'!$I$11</x:f>
-        <x:v>82888639.97287165</x:v>
+        <x:v>41444319.98643582</x:v>
       </x:c>
       <x:c r="J17" s="34" t="n">
         <x:f>MIN(1,I17/'Assumptions'!$B$9)</x:f>
-        <x:v>0.48359766611943783</x:v>
+        <x:v>0.24179883305971892</x:v>
       </x:c>
       <x:c r="K17" s="34" t="n">
         <x:f>J17-J16</x:f>
-        <x:v>0.10772041382327108</x:v>
+        <x:v>0.05386020691163554</x:v>
       </x:c>
       <x:c r="L17" s="23" t="str">
         <x:f>IF(J17&gt;='Assumptions'!$G$16,"A",IF(J17&gt;='Assumptions'!$G$17,"B",IF(J17&gt;='Assumptions'!$G$18,"C",IF(J17&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3274,19 +3274,19 @@
       </x:c>
       <x:c r="H18" s="33" t="n">
         <x:f>E18*'Assumptions'!$B$25</x:f>
-        <x:v>1625234633809920</x:v>
+        <x:v>812617316904960</x:v>
       </x:c>
       <x:c r="I18" s="29" t="n">
         <x:f>H18/'Assumptions'!$I$11</x:f>
-        <x:v>97028933.36178628</x:v>
+        <x:v>48514466.68089314</x:v>
       </x:c>
       <x:c r="J18" s="34" t="n">
         <x:f>MIN(1,I18/'Assumptions'!$B$9)</x:f>
-        <x:v>0.5660964606872011</x:v>
+        <x:v>0.28304823034360055</x:v>
       </x:c>
       <x:c r="K18" s="34" t="n">
         <x:f>J18-J17</x:f>
-        <x:v>0.08249879456776327</x:v>
+        <x:v>0.041249397283881634</x:v>
       </x:c>
       <x:c r="L18" s="23" t="str">
         <x:f>IF(J18&gt;='Assumptions'!$G$16,"A",IF(J18&gt;='Assumptions'!$G$17,"B",IF(J18&gt;='Assumptions'!$G$18,"C",IF(J18&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3324,19 +3324,19 @@
       </x:c>
       <x:c r="H19" s="33" t="n">
         <x:f>E19*'Assumptions'!$B$25</x:f>
-        <x:v>1710711429557760</x:v>
+        <x:v>855355714778880</x:v>
       </x:c>
       <x:c r="I19" s="29" t="n">
         <x:f>H19/'Assumptions'!$I$11</x:f>
-        <x:v>102132025.6452394</x:v>
+        <x:v>51066012.8226197</x:v>
       </x:c>
       <x:c r="J19" s="34" t="n">
         <x:f>MIN(1,I19/'Assumptions'!$B$9)</x:f>
-        <x:v>0.5958694611740921</x:v>
+        <x:v>0.29793473058704606</x:v>
       </x:c>
       <x:c r="K19" s="34" t="n">
         <x:f>J19-J18</x:f>
-        <x:v>0.02977300048689102</x:v>
+        <x:v>0.01488650024344551</x:v>
       </x:c>
       <x:c r="L19" s="23" t="str">
         <x:f>IF(J19&gt;='Assumptions'!$G$16,"A",IF(J19&gt;='Assumptions'!$G$17,"B",IF(J19&gt;='Assumptions'!$G$18,"C",IF(J19&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3374,27 +3374,27 @@
       </x:c>
       <x:c r="H20" s="33" t="n">
         <x:f>E20*'Assumptions'!$B$25</x:f>
-        <x:v>1854584618100480</x:v>
+        <x:v>927292309050240</x:v>
       </x:c>
       <x:c r="I20" s="29" t="n">
         <x:f>H20/'Assumptions'!$I$11</x:f>
-        <x:v>110721469.73734209</x:v>
+        <x:v>55360734.868671045</x:v>
       </x:c>
       <x:c r="J20" s="34" t="n">
         <x:f>MIN(1,I20/'Assumptions'!$B$9)</x:f>
-        <x:v>0.6459829039518208</x:v>
+        <x:v>0.3229914519759104</x:v>
       </x:c>
       <x:c r="K20" s="34" t="n">
         <x:f>J20-J19</x:f>
-        <x:v>0.05011344277772867</x:v>
+        <x:v>0.025056721388864334</x:v>
       </x:c>
       <x:c r="L20" s="23" t="str">
         <x:f>IF(J20&gt;='Assumptions'!$G$16,"A",IF(J20&gt;='Assumptions'!$G$17,"B",IF(J20&gt;='Assumptions'!$G$18,"C",IF(J20&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
-        <x:v>D</x:v>
+        <x:v>F</x:v>
       </x:c>
       <x:c r="M20" s="35" t="n">
         <x:f>IF(J20&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J20&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J20&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J20&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -3424,27 +3424,27 @@
       </x:c>
       <x:c r="H21" s="33" t="n">
         <x:f>E21*'Assumptions'!$B$25</x:f>
-        <x:v>2398401754116480</x:v>
+        <x:v>1199200877058240</x:v>
       </x:c>
       <x:c r="I21" s="29" t="n">
         <x:f>H21/'Assumptions'!$I$11</x:f>
-        <x:v>143188164.42486447</x:v>
+        <x:v>71594082.21243224</x:v>
       </x:c>
       <x:c r="J21" s="34" t="n">
         <x:f>MIN(1,I21/'Assumptions'!$B$9)</x:f>
-        <x:v>0.8354035263994427</x:v>
+        <x:v>0.41770176319972135</x:v>
       </x:c>
       <x:c r="K21" s="34" t="n">
         <x:f>J21-J20</x:f>
-        <x:v>0.18942062244762192</x:v>
+        <x:v>0.09471031122381096</x:v>
       </x:c>
       <x:c r="L21" s="23" t="str">
         <x:f>IF(J21&gt;='Assumptions'!$G$16,"A",IF(J21&gt;='Assumptions'!$G$17,"B",IF(J21&gt;='Assumptions'!$G$18,"C",IF(J21&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
-        <x:v>B</x:v>
+        <x:v>F</x:v>
       </x:c>
       <x:c r="M21" s="35" t="n">
         <x:f>IF(J21&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J21&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J21&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J21&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -3474,27 +3474,27 @@
       </x:c>
       <x:c r="H22" s="33" t="n">
         <x:f>E22*'Assumptions'!$B$25</x:f>
-        <x:v>2956200827207040</x:v>
+        <x:v>1478100413603520</x:v>
       </x:c>
       <x:c r="I22" s="29" t="n">
         <x:f>H22/'Assumptions'!$I$11</x:f>
-        <x:v>176489601.6243009</x:v>
+        <x:v>88244800.81215045</x:v>
       </x:c>
       <x:c r="J22" s="34" t="n">
         <x:f>MIN(1,I22/'Assumptions'!$B$9)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.5148471459285324</x:v>
       </x:c>
       <x:c r="K22" s="34" t="n">
         <x:f>J22-J21</x:f>
-        <x:v>0.1645964736005573</x:v>
+        <x:v>0.09714538272881107</x:v>
       </x:c>
       <x:c r="L22" s="23" t="str">
         <x:f>IF(J22&gt;='Assumptions'!$G$16,"A",IF(J22&gt;='Assumptions'!$G$17,"B",IF(J22&gt;='Assumptions'!$G$18,"C",IF(J22&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
-        <x:v>A</x:v>
+        <x:v>F</x:v>
       </x:c>
       <x:c r="M22" s="35" t="n">
         <x:f>IF(J22&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J22&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J22&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J22&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
@@ -3524,27 +3524,27 @@
       </x:c>
       <x:c r="H23" s="33" t="n">
         <x:f>E23*'Assumptions'!$B$25</x:f>
-        <x:v>3673493660712960</x:v>
+        <x:v>1836746830356480</x:v>
       </x:c>
       <x:c r="I23" s="29" t="n">
         <x:f>H23/'Assumptions'!$I$11</x:f>
-        <x:v>219313054.37092298</x:v>
+        <x:v>109656527.18546149</x:v>
       </x:c>
       <x:c r="J23" s="34" t="n">
         <x:f>MIN(1,I23/'Assumptions'!$B$9)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.6397697035324474</x:v>
       </x:c>
       <x:c r="K23" s="34" t="n">
         <x:f>J23-J22</x:f>
-        <x:v>0</x:v>
+        <x:v>0.12492255760391502</x:v>
       </x:c>
       <x:c r="L23" s="23" t="str">
         <x:f>IF(J23&gt;='Assumptions'!$G$16,"A",IF(J23&gt;='Assumptions'!$G$17,"B",IF(J23&gt;='Assumptions'!$G$18,"C",IF(J23&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
-        <x:v>A</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="M23" s="35" t="n">
         <x:f>IF(J23&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J23&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J23&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J23&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
@@ -3574,27 +3574,27 @@
       </x:c>
       <x:c r="H24" s="33" t="n">
         <x:f>E24*'Assumptions'!$B$25</x:f>
-        <x:v>3758810790107520</x:v>
+        <x:v>1879405395053760</x:v>
       </x:c>
       <x:c r="I24" s="29" t="n">
         <x:f>H24/'Assumptions'!$I$11</x:f>
-        <x:v>224406614.33477733</x:v>
+        <x:v>112203307.16738866</x:v>
       </x:c>
       <x:c r="J24" s="34" t="n">
         <x:f>MIN(1,I24/'Assumptions'!$B$9)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.6546283965425242</x:v>
       </x:c>
       <x:c r="K24" s="34" t="n">
         <x:f>J24-J23</x:f>
-        <x:v>0</x:v>
+        <x:v>0.014858693010076807</x:v>
       </x:c>
       <x:c r="L24" s="23" t="str">
         <x:f>IF(J24&gt;='Assumptions'!$G$16,"A",IF(J24&gt;='Assumptions'!$G$17,"B",IF(J24&gt;='Assumptions'!$G$18,"C",IF(J24&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
-        <x:v>A</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="M24" s="35" t="n">
         <x:f>IF(J24&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J24&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J24&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J24&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
@@ -3624,27 +3624,27 @@
       </x:c>
       <x:c r="H25" s="33" t="n">
         <x:f>E25*'Assumptions'!$B$25</x:f>
-        <x:v>4938170788817280</x:v>
+        <x:v>2469085394408640</x:v>
       </x:c>
       <x:c r="I25" s="29" t="n">
         <x:f>H25/'Assumptions'!$I$11</x:f>
-        <x:v>294816166.496554</x:v>
+        <x:v>147408083.248277</x:v>
       </x:c>
       <x:c r="J25" s="34" t="n">
         <x:f>MIN(1,I25/'Assumptions'!$B$9)</x:f>
-        <x:v>1</x:v>
+        <x:v>0.860023822918769</x:v>
       </x:c>
       <x:c r="K25" s="34" t="n">
         <x:f>J25-J24</x:f>
-        <x:v>0</x:v>
+        <x:v>0.20539542637624475</x:v>
       </x:c>
       <x:c r="L25" s="23" t="str">
         <x:f>IF(J25&gt;='Assumptions'!$G$16,"A",IF(J25&gt;='Assumptions'!$G$17,"B",IF(J25&gt;='Assumptions'!$G$18,"C",IF(J25&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="M25" s="35" t="n">
         <x:f>IF(J25&gt;='Assumptions'!$G$16,'Assumptions'!$H$16,IF(J25&gt;='Assumptions'!$G$17,'Assumptions'!$H$17,IF(J25&gt;='Assumptions'!$G$18,'Assumptions'!$H$18,IF(J25&gt;='Assumptions'!$G$19,'Assumptions'!$H$19,'Assumptions'!$H$20))))</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3654,7 +3654,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1aa90f741855464a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca38904d8b934203"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3952,7 +3952,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>B9*I11/B25</x:f>
-        <x:v>35979846.92445279</x:v>
+        <x:v>71959693.84890558</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>H100e</x:v>
@@ -4170,7 +4170,7 @@
         <x:v>Personal-AI share of modeled inference</x:v>
       </x:c>
       <x:c r="B24" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="C24" s="17" t="str">
         <x:v>%</x:v>
@@ -4185,7 +4185,7 @@
       </x:c>
       <x:c r="B25" s="18" t="n">
         <x:f>B16*B17*B18*B19*B23*B24/(B20*B21*B22)</x:f>
-        <x:v>79793280</x:v>
+        <x:v>39896640</x:v>
       </x:c>
       <x:c r="C25" s="17" t="str">
         <x:v>tokens/day</x:v>
@@ -4267,34 +4267,34 @@
         <x:v>Growth from the current snapshot to 2026-Q4</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="15" hidden="0" customHeight="1">
+    <x:row r="31" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A31" s="17" t="str">
         <x:v>First model row at full supply threshold</x:v>
       </x:c>
-      <x:c r="B31" s="17" t="n">
-        <x:f>MATCH(1,'Quarterly Model'!$J$6:$J$25,0)</x:f>
-        <x:v>17</x:v>
+      <x:c r="B31" s="17" t="str">
+        <x:f>IFERROR(MATCH(1,'Quarterly Model'!$J$6:$J$25,0),"Beyond window")</x:f>
+        <x:v>Beyond window</x:v>
       </x:c>
       <x:c r="C31" s="17" t="str">
         <x:v>position</x:v>
       </x:c>
       <x:c r="D31" s="17" t="str">
-        <x:v>First score that reaches 100%</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="15" hidden="0" customHeight="1">
+        <x:v>First score that reaches 100%; 'Beyond window' when extrapolation is required</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A32" s="17" t="str">
         <x:v>Projected supply crossing</x:v>
       </x:c>
       <x:c r="B32" s="20" t="n">
-        <x:f>INDEX('Quarterly Model'!$C$6:$C$25,B31-1)+(B12-INDEX('Quarterly Model'!$E$6:$E$25,B31-1))/(INDEX('Quarterly Model'!$E$6:$E$25,B31)-INDEX('Quarterly Model'!$E$6:$E$25,B31-1))*(INDEX('Quarterly Model'!$C$6:$C$25,B31)-INDEX('Quarterly Model'!$C$6:$C$25,B31-1))</x:f>
-        <x:v>46829.09207929863</x:v>
+        <x:f>IF(ISNUMBER(B31),INDEX('Quarterly Model'!$C$6:$C$25,B31-1)+(B12-INDEX('Quarterly Model'!$E$6:$E$25,B31-1))/(INDEX('Quarterly Model'!$E$6:$E$25,B31)-INDEX('Quarterly Model'!$E$6:$E$25,B31-1))*(INDEX('Quarterly Model'!$C$6:$C$25,B31)-INDEX('Quarterly Model'!$C$6:$C$25,B31-1)),'Quarterly Model'!$C$25+IF(ABS(B28)&lt;0.000000001,(LN(B12/'Quarterly Model'!$E$25)/LN(2))/'Quarterly Model'!$G$25,(-('Quarterly Model'!$G$25+B28/2)+SQRT(('Quarterly Model'!$G$25+B28/2)^2-2*B28*(LN('Quarterly Model'!$E$25/B12)/LN(2))))/B28)*(365.2425/4))</x:f>
+        <x:v>47168.12398813577</x:v>
       </x:c>
       <x:c r="C32" s="17" t="str">
         <x:v>date</x:v>
       </x:c>
       <x:c r="D32" s="17" t="str">
-        <x:v>Linear interpolation between surrounding capacity points</x:v>
+        <x:v>Interpolate inside the report window; otherwise extend the final log-growth velocity and pipeline acceleration</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
@@ -4331,7 +4331,7 @@
       </x:c>
       <x:c r="B35" s="20" t="n">
         <x:f>MAX(B32,B34)</x:f>
-        <x:v>46924</x:v>
+        <x:v>47168.12398813577</x:v>
       </x:c>
       <x:c r="C35" s="17" t="str">
         <x:v>date</x:v>
@@ -4927,7 +4927,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5990f97ea774270"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc36f2a52061145b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5152,7 +5152,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd156bc7772fb4a2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b14c28f2b594f4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Model recursive progress feedback
</commit_message>
<xml_diff>
--- a/data/reports/personal-ai-compute-report-card.xlsx
+++ b/data/reports/personal-ai-compute-report-card.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4ad33934139b4500"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compute Report Card" sheetId="2" r:id="Re98b9d51da3d4e8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="3" r:id="R48a1feb01b7345b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Ra4938a3d59374b6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" r:id="R368602b363824e18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R0a5e5e32eebd45b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rfc382ce6611a4867"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compute Report Card" sheetId="2" r:id="R72c0a8b1b13c4935"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="3" r:id="R51fce068a25f4f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R0c209b41f52345d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" r:id="Rdf2de95b6b3d400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Ra758f9754477402f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -470,7 +470,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc5bdbe21adb0459a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3f0d0dbe41ca49cb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -934,7 +934,7 @@
       </x:c>
       <x:c r="J6" s="58" t="n">
         <x:f>'Assumptions'!B32</x:f>
-        <x:v>47168.12398813577</x:v>
+        <x:v>47168.337489406</x:v>
       </x:c>
       <x:c r="M6" s="54" t="str">
         <x:f>'Quarterly Model'!L16</x:f>
@@ -996,7 +996,7 @@
         <x:v>0.45660533834944794</x:v>
       </x:c>
       <x:c r="D13" s="20" t="n">
-        <x:v>46924</x:v>
+        <x:v>46502</x:v>
       </x:c>
       <x:c r="E13" s="17" t="str">
         <x:v>Waiting</x:v>
@@ -1018,7 +1018,7 @@
       </x:c>
       <x:c r="D14" s="20" t="n">
         <x:f>'Assumptions'!B32</x:f>
-        <x:v>47168.12398813577</x:v>
+        <x:v>47168.337489406</x:v>
       </x:c>
       <x:c r="E14" s="17" t="str">
         <x:v>Waiting</x:v>
@@ -1037,7 +1037,7 @@
       <x:c r="C15" s="24"/>
       <x:c r="D15" s="59" t="n">
         <x:f>'Assumptions'!B35</x:f>
-        <x:v>47168.12398813577</x:v>
+        <x:v>47168.337489406</x:v>
       </x:c>
       <x:c r="E15" s="24" t="str">
         <x:v>Later crossing</x:v>
@@ -1376,7 +1376,7 @@
         <x:v>Projection</x:v>
       </x:c>
       <x:c r="B42" s="17" t="str">
-        <x:v>The base path sums dated expected or projected operating states in Epoch's current U.S. buildout timeline. The displayed acceleration is descriptive of that source path, not a fitted causal law.</x:v>
+        <x:v>The base path sums dated expected or projected operating states in Epoch's current U.S. buildout timeline. Beyond that window, log-growth follows dv/dh = k·v with k = acceleration / velocity; this causal feedback is a scenario assumption.</x:v>
       </x:c>
       <x:c r="C42" s="17"/>
       <x:c r="D42" s="17"/>
@@ -1453,7 +1453,7 @@
     <x:mergeCell ref="B44:N44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2acf7977cf74b65"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb497740d07a2427a"/>
 </x:worksheet>
 </file>
 
@@ -2417,7 +2417,7 @@
       </x:c>
       <x:c r="AT6" s="20" t="n">
         <x:f>'Assumptions'!B32</x:f>
-        <x:v>47168.12398813577</x:v>
+        <x:v>47168.337489406</x:v>
       </x:c>
       <x:c r="AU6" s="27" t="n">
         <x:f>'Assumptions'!B30</x:f>
@@ -3654,7 +3654,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca38904d8b934203"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc72a9ba6d26448e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4287,14 +4287,14 @@
         <x:v>Projected supply crossing</x:v>
       </x:c>
       <x:c r="B32" s="20" t="n">
-        <x:f>IF(ISNUMBER(B31),INDEX('Quarterly Model'!$C$6:$C$25,B31-1)+(B12-INDEX('Quarterly Model'!$E$6:$E$25,B31-1))/(INDEX('Quarterly Model'!$E$6:$E$25,B31)-INDEX('Quarterly Model'!$E$6:$E$25,B31-1))*(INDEX('Quarterly Model'!$C$6:$C$25,B31)-INDEX('Quarterly Model'!$C$6:$C$25,B31-1)),'Quarterly Model'!$C$25+IF(ABS(B28)&lt;0.000000001,(LN(B12/'Quarterly Model'!$E$25)/LN(2))/'Quarterly Model'!$G$25,(-('Quarterly Model'!$G$25+B28/2)+SQRT(('Quarterly Model'!$G$25+B28/2)^2-2*B28*(LN('Quarterly Model'!$E$25/B12)/LN(2))))/B28)*(365.2425/4))</x:f>
-        <x:v>47168.12398813577</x:v>
+        <x:f>IF(ISNUMBER(B31),INDEX('Quarterly Model'!$C$6:$C$25,B31-1)+(B12-INDEX('Quarterly Model'!$E$6:$E$25,B31-1))/(INDEX('Quarterly Model'!$E$6:$E$25,B31)-INDEX('Quarterly Model'!$E$6:$E$25,B31-1))*(INDEX('Quarterly Model'!$C$6:$C$25,B31)-INDEX('Quarterly Model'!$C$6:$C$25,B31-1)),'Quarterly Model'!$C$25+IF(ABS(B28)&lt;0.000000001,(LN(B12/'Quarterly Model'!$E$25)/LN(2))/'Quarterly Model'!$G$25,IF(1+(B28/'Quarterly Model'!$G$25)*(LN(B12/'Quarterly Model'!$E$25)/LN(2))/'Quarterly Model'!$G$25&lt;=0,NA(),LN(1+(B28/'Quarterly Model'!$G$25)*(LN(B12/'Quarterly Model'!$E$25)/LN(2))/'Quarterly Model'!$G$25)/(B28/'Quarterly Model'!$G$25)))*(365.2425/4))</x:f>
+        <x:v>47168.337489406</x:v>
       </x:c>
       <x:c r="C32" s="17" t="str">
         <x:v>date</x:v>
       </x:c>
       <x:c r="D32" s="17" t="str">
-        <x:v>Interpolate inside the report window; otherwise extend the final log-growth velocity and pipeline acceleration</x:v>
+        <x:v>Interpolate inside the report window; otherwise use dv/dh = k·v with k = acceleration / velocity</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
@@ -4316,13 +4316,13 @@
         <x:v>Projected capability crossing</x:v>
       </x:c>
       <x:c r="B34" s="20" t="n">
-        <x:v>46924</x:v>
+        <x:v>46502</x:v>
       </x:c>
       <x:c r="C34" s="17" t="str">
         <x:v>date</x:v>
       </x:c>
       <x:c r="D34" s="17" t="str">
-        <x:v>First UTC day on which the capability report-card path reaches 60%</x:v>
+        <x:v>First UTC day on which the shared-frontier capability path reaches 60%</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
@@ -4331,7 +4331,7 @@
       </x:c>
       <x:c r="B35" s="20" t="n">
         <x:f>MAX(B32,B34)</x:f>
-        <x:v>47168.12398813577</x:v>
+        <x:v>47168.337489406</x:v>
       </x:c>
       <x:c r="C35" s="17" t="str">
         <x:v>date</x:v>
@@ -4927,7 +4927,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc36f2a52061145b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63ea93586e2f4266"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5142,7 +5142,7 @@
         <x:v>https://diffuse-personal-ai-countdown.buddywilliams.chatgpt.site/?report=capability</x:v>
       </x:c>
       <x:c r="F11" s="17" t="str">
-        <x:v>Capability first reaches 60% on the daily site path on 2028-06-20</x:v>
+        <x:v>Capability first reaches 60% on the daily shared-frontier path on 2027-04-25</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5152,7 +5152,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b14c28f2b594f4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcabf2cc9bd8c49ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Model capability acceleration with METR horizons
</commit_message>
<xml_diff>
--- a/data/reports/personal-ai-compute-report-card.xlsx
+++ b/data/reports/personal-ai-compute-report-card.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rfc382ce6611a4867"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compute Report Card" sheetId="2" r:id="R72c0a8b1b13c4935"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="3" r:id="R51fce068a25f4f88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R0c209b41f52345d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" r:id="Rdf2de95b6b3d400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Ra758f9754477402f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re1ab6de16dd84ebc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compute Report Card" sheetId="2" r:id="Rb321fecbf4054aa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="3" r:id="Rbb329da357ae40a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rb49b49762f224e2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" r:id="Rd42d5c52781745c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R02d37d2892d749f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -470,7 +470,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3f0d0dbe41ca49cb"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf7a4042ff74a44e1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -990,13 +990,13 @@
         <x:v>Demand / capability</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>Capability report ≥60%</x:v>
+        <x:v>Capability report ≥75%</x:v>
       </x:c>
       <x:c r="C13" s="31" t="n">
         <x:v>0.45660533834944794</x:v>
       </x:c>
       <x:c r="D13" s="20" t="n">
-        <x:v>46502</x:v>
+        <x:v>46704</x:v>
       </x:c>
       <x:c r="E13" s="17" t="str">
         <x:v>Waiting</x:v>
@@ -1453,7 +1453,7 @@
     <x:mergeCell ref="B44:N44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb497740d07a2427a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9566bceff9884382"/>
 </x:worksheet>
 </file>
 
@@ -3654,7 +3654,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc72a9ba6d26448e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b934f6f0ebf4067"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4302,27 +4302,27 @@
         <x:v>Capability threshold</x:v>
       </x:c>
       <x:c r="B33" s="19" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="C33" s="17" t="str">
         <x:v>%</x:v>
       </x:c>
       <x:c r="D33" s="17" t="str">
-        <x:v>First grade above F</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="15" hidden="0" customHeight="1">
+        <x:v>Default practical delegation-quality gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A34" s="17" t="str">
         <x:v>Projected capability crossing</x:v>
       </x:c>
       <x:c r="B34" s="20" t="n">
-        <x:v>46502</x:v>
+        <x:v>46704</x:v>
       </x:c>
       <x:c r="C34" s="17" t="str">
         <x:v>date</x:v>
       </x:c>
       <x:c r="D34" s="17" t="str">
-        <x:v>First UTC day on which the shared-frontier capability path reaches 60%</x:v>
+        <x:v>First UTC day on which the economic benchmark path with METR H50/H80 feedback reaches 75%</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
@@ -4927,7 +4927,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63ea93586e2f4266"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55b7b9aae5084660"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5125,7 +5125,7 @@
         <x:v>Serving envelope and high-autonomy token mix; assumptions remain editable</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
+    <x:row r="11" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A11" s="17" t="str">
         <x:v>SRC-006</x:v>
       </x:c>
@@ -5142,7 +5142,7 @@
         <x:v>https://diffuse-personal-ai-countdown.buddywilliams.chatgpt.site/?report=capability</x:v>
       </x:c>
       <x:c r="F11" s="17" t="str">
-        <x:v>Capability first reaches 60% on the daily shared-frontier path on 2027-04-25</x:v>
+        <x:v>Capability first reaches 75% on the daily economic benchmark path with METR H50/H80 feedback on 2027-11-13</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5152,7 +5152,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcabf2cc9bd8c49ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c1eb75459764854"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>